<commit_message>
fix: close v0.3 review findings
</commit_message>
<xml_diff>
--- a/outputs/v0.3-review/production-system-model-template-v0.3-review.xlsx
+++ b/outputs/v0.3-review/production-system-model-template-v0.3-review.xlsx
@@ -2,39 +2,84 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R25561d67367e4b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Система" sheetId="2" r:id="Rbb537b34a2264001"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Схема шаблона" sheetId="3" r:id="R114402b29e3c44c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="4" r:id="Rce9bfce3f0e742fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версии" sheetId="5" r:id="R4e7290eb8c7d4cd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исполнители" sheetId="6" r:id="R6095b1044e23474e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции" sheetId="7" r:id="R2a762e366ecc41a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Назначения" sheetId="8" r:id="Rca2507f0dc304c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контрагенты" sheetId="9" r:id="Re083bdc365da41bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Продукты" sheetId="10" r:id="R76f58e688ec34110"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Материалы" sheetId="11" r:id="R0b18ec3db8ac4d4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процессы" sheetId="12" r:id="R625b236fa3e64313"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действия" sheetId="13" r:id="R5ffe72163fc54f1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи действий" sheetId="14" r:id="R1673c2d81d07498a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объекты" sheetId="15" r:id="R79ac09509a2b4a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Состояния" sheetId="16" r:id="Rdde3ba16211f41bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переходы" sheetId="17" r:id="R6cdc730a97664e7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Элементы модели" sheetId="18" r:id="R24321080cd0142e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контракты" sheetId="19" r:id="R0122902d900d4ca8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции контрактов" sheetId="20" r:id="R13e6b99705b64ff6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Интерфейсы передачи" sheetId="21" r:id="Ra3de342306734aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи модели" sheetId="22" r:id="Rdf1e01892b684fd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Решения" sheetId="23" r:id="Re8918e4eeb7340b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения модели" sheetId="24" r:id="R82b27728037847d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отклонения" sheetId="25" r:id="R24cf50b5a0eb4dc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гипотезы" sheetId="26" r:id="Rac39fea5acfc4a30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперименты" sheetId="27" r:id="Rb249abd9af584c4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез модели" sheetId="28" r:id="R124b2d56719e48c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Проверки" sheetId="29" r:id="R80096a28dd4f441d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр процессов" sheetId="30" r:id="Ra585cd61409542d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Рабочая панель" sheetId="31" r:id="Rdb94449ea907430d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Диаграммы" sheetId="32" r:id="R47973f9b30364307"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R0b3dca1709464630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Система" sheetId="2" r:id="Re60b5d214226498c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Схема шаблона" sheetId="3" r:id="R80280a7af63a4d22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="4" r:id="Rb9187a0402fe439b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версии" sheetId="5" r:id="R7ca2923ced694aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исполнители" sheetId="6" r:id="R73e6818c8eb44a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции" sheetId="7" r:id="Rbbe6743c120a4aad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Назначения" sheetId="8" r:id="R4c506565d622472f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контрагенты" sheetId="9" r:id="Re705a6aad1b54082"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Продукты" sheetId="10" r:id="R505d702d6be84e27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Материалы" sheetId="11" r:id="Rdd94ab43ccff4e45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процессы" sheetId="12" r:id="R0ff262c936e3422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действия" sheetId="13" r:id="R3b39098b32004a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи действий" sheetId="14" r:id="R62c6000634514408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объекты" sheetId="15" r:id="R3a35579690bf4a6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Состояния" sheetId="16" r:id="R87f28f98d0eb4900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переходы" sheetId="17" r:id="R511d0ff9eef24b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Элементы модели" sheetId="18" r:id="R0dea83fddd074536"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контракты" sheetId="19" r:id="R986026adf49b4020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции контрактов" sheetId="20" r:id="Rcebfd67ffefa4517"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Интерфейсы передачи" sheetId="21" r:id="R239056d14fe743e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи модели" sheetId="22" r:id="Rcc64aaaba5e34cbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Решения" sheetId="23" r:id="Rad6d7730ddb2452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения модели" sheetId="24" r:id="Rd7d8078d8e2148eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отклонения" sheetId="25" r:id="R3e09a0ff3486487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гипотезы" sheetId="26" r:id="Rdebf444f9856493e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперименты" sheetId="27" r:id="Ra722a18f03424663"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез модели" sheetId="28" r:id="Rb1851d1b039c4976"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Проверки" sheetId="29" r:id="R4cbafd61b3aa4a9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр процессов" sheetId="30" r:id="R80f9f697e22f4c76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Рабочая панель" sheetId="31" r:id="R1ec4699c29e44e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Диаграммы" sheetId="32" r:id="R53c3ac159ab243c1"/>
   </x:sheets>
+  <x:definedNames>
+    <x:definedName name="enum_yes_no">'Система'!BA2:BA3</x:definedName>
+    <x:definedName name="enum_version_operation">'Система'!BB2:BB3</x:definedName>
+    <x:definedName name="enum_knowledge_status">'Система'!BC2:BC7</x:definedName>
+    <x:definedName name="enum_model_layer">'Система'!BD2:BD3</x:definedName>
+    <x:definedName name="enum_version_status">'Система'!BE2:BE5</x:definedName>
+    <x:definedName name="enum_execution_status">'Система'!BF2:BF5</x:definedName>
+    <x:definedName name="enum_performer_type">'Система'!BG2:BG3</x:definedName>
+    <x:definedName name="enum_assignment_status">'Система'!BH2:BH4</x:definedName>
+    <x:definedName name="enum_counterparty_type">'Система'!BI2:BI3</x:definedName>
+    <x:definedName name="enum_action_type">'Система'!BJ2:BJ7</x:definedName>
+    <x:definedName name="enum_performer_mode">'Система'!BK2:BK5</x:definedName>
+    <x:definedName name="enum_edge_type">'Система'!BL2:BL6</x:definedName>
+    <x:definedName name="enum_object_type">'Система'!BM2:BM7</x:definedName>
+    <x:definedName name="enum_element_type">'Система'!BN2:BN11</x:definedName>
+    <x:definedName name="enum_contract_status">'Система'!BO2:BO5</x:definedName>
+    <x:definedName name="enum_direction">'Система'!BP2:BP3</x:definedName>
+    <x:definedName name="enum_pricing_method">'Система'!BQ2:BQ5</x:definedName>
+    <x:definedName name="enum_change_operation">'Система'!BR2:BR6</x:definedName>
+    <x:definedName name="enum_projection_kind">'Система'!BS2:BS3</x:definedName>
+    <x:definedName name="enum_readiness_status">'Система'!BT2:BT4</x:definedName>
+    <x:definedName name="enum_resolution_status">'Система'!BU2:BU4</x:definedName>
+    <x:definedName name="enum_check_severity">'Система'!BV2:BV4</x:definedName>
+    <x:definedName name="enum_development_scope_type">'Система'!BW2:BW9</x:definedName>
+    <x:definedName name="enum_deviation_status">'Система'!BX2:BX7</x:definedName>
+    <x:definedName name="enum_deviation_type">'Система'!BY2:BY5</x:definedName>
+    <x:definedName name="enum_evidence_channel">'Система'!BZ2:BZ3</x:definedName>
+    <x:definedName name="enum_cause_status">'Система'!CA2:CA4</x:definedName>
+    <x:definedName name="enum_verification_status">'Система'!CB2:CB5</x:definedName>
+    <x:definedName name="enum_hypothesis_status">'Система'!CC2:CC6</x:definedName>
+    <x:definedName name="enum_evidence_result">'Система'!CD2:CD4</x:definedName>
+    <x:definedName name="enum_development_decision">'Система'!CE2:CE4</x:definedName>
+    <x:definedName name="enum_experiment_status">'Система'!CF2:CF7</x:definedName>
+    <x:definedName name="enum_experiment_basis_type">'Система'!CG2:CG3</x:definedName>
+    <x:definedName name="selector_demo_versions">'Система'!CH1:CH1</x:definedName>
+    <x:definedName name="selector_demo_versions_ids">'Система'!CI1:CI1</x:definedName>
+    <x:definedName name="selector_demo_systems">'Система'!CJ1:CJ1</x:definedName>
+    <x:definedName name="selector_demo_systems_ids">'Система'!CK1:CK1</x:definedName>
+    <x:definedName name="selector_demo_processes">'Система'!CL1:CL1</x:definedName>
+    <x:definedName name="selector_demo_processes_ids">'Система'!CM1:CM1</x:definedName>
+    <x:definedName name="selector_demo_positions">'Система'!CN1:CN1</x:definedName>
+    <x:definedName name="selector_demo_positions_ids">'Система'!CO1:CO1</x:definedName>
+    <x:definedName name="selector_demo_metrics">'Система'!CP1:CP1</x:definedName>
+    <x:definedName name="selector_demo_metrics_ids">'Система'!CQ1:CQ1</x:definedName>
+  </x:definedNames>
 </x:workbook>
 </file>
 
@@ -254,6 +299,19 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="1">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A1C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
@@ -22099,6 +22157,135 @@
       <x:c r="L1" s="16"/>
       <x:c r="M1" s="2"/>
       <x:c r="N1" s="2"/>
+      <x:c r="BA1" t="str">
+        <x:v>yes_no</x:v>
+      </x:c>
+      <x:c r="BB1" t="str">
+        <x:v>version_operation</x:v>
+      </x:c>
+      <x:c r="BC1" t="str">
+        <x:v>knowledge_status</x:v>
+      </x:c>
+      <x:c r="BD1" t="str">
+        <x:v>model_layer</x:v>
+      </x:c>
+      <x:c r="BE1" t="str">
+        <x:v>version_status</x:v>
+      </x:c>
+      <x:c r="BF1" t="str">
+        <x:v>execution_status</x:v>
+      </x:c>
+      <x:c r="BG1" t="str">
+        <x:v>performer_type</x:v>
+      </x:c>
+      <x:c r="BH1" t="str">
+        <x:v>assignment_status</x:v>
+      </x:c>
+      <x:c r="BI1" t="str">
+        <x:v>counterparty_type</x:v>
+      </x:c>
+      <x:c r="BJ1" t="str">
+        <x:v>action_type</x:v>
+      </x:c>
+      <x:c r="BK1" t="str">
+        <x:v>performer_mode</x:v>
+      </x:c>
+      <x:c r="BL1" t="str">
+        <x:v>edge_type</x:v>
+      </x:c>
+      <x:c r="BM1" t="str">
+        <x:v>object_type</x:v>
+      </x:c>
+      <x:c r="BN1" t="str">
+        <x:v>element_type</x:v>
+      </x:c>
+      <x:c r="BO1" t="str">
+        <x:v>contract_status</x:v>
+      </x:c>
+      <x:c r="BP1" t="str">
+        <x:v>direction</x:v>
+      </x:c>
+      <x:c r="BQ1" t="str">
+        <x:v>pricing_method</x:v>
+      </x:c>
+      <x:c r="BR1" t="str">
+        <x:v>change_operation</x:v>
+      </x:c>
+      <x:c r="BS1" t="str">
+        <x:v>projection_kind</x:v>
+      </x:c>
+      <x:c r="BT1" t="str">
+        <x:v>readiness_status</x:v>
+      </x:c>
+      <x:c r="BU1" t="str">
+        <x:v>resolution_status</x:v>
+      </x:c>
+      <x:c r="BV1" t="str">
+        <x:v>check_severity</x:v>
+      </x:c>
+      <x:c r="BW1" t="str">
+        <x:v>development_scope_type</x:v>
+      </x:c>
+      <x:c r="BX1" t="str">
+        <x:v>deviation_status</x:v>
+      </x:c>
+      <x:c r="BY1" t="str">
+        <x:v>deviation_type</x:v>
+      </x:c>
+      <x:c r="BZ1" t="str">
+        <x:v>evidence_channel</x:v>
+      </x:c>
+      <x:c r="CA1" t="str">
+        <x:v>cause_status</x:v>
+      </x:c>
+      <x:c r="CB1" t="str">
+        <x:v>verification_status</x:v>
+      </x:c>
+      <x:c r="CC1" t="str">
+        <x:v>hypothesis_status</x:v>
+      </x:c>
+      <x:c r="CD1" t="str">
+        <x:v>evidence_result</x:v>
+      </x:c>
+      <x:c r="CE1" t="str">
+        <x:v>development_decision</x:v>
+      </x:c>
+      <x:c r="CF1" t="str">
+        <x:v>experiment_status</x:v>
+      </x:c>
+      <x:c r="CG1" t="str">
+        <x:v>experiment_basis_type</x:v>
+      </x:c>
+      <x:c r="CH1" t="str">
+        <x:v>Текущая модель v0.3</x:v>
+      </x:c>
+      <x:c r="CI1" t="str">
+        <x:v>ver-demo-v0.3</x:v>
+      </x:c>
+      <x:c r="CJ1" t="str">
+        <x:v>Привлечение</x:v>
+      </x:c>
+      <x:c r="CK1" t="str">
+        <x:v>ps-demo-attraction</x:v>
+      </x:c>
+      <x:c r="CL1" t="str">
+        <x:v>Обработка лида</x:v>
+      </x:c>
+      <x:c r="CM1" t="str">
+        <x:v>prc-demo-lead</x:v>
+      </x:c>
+      <x:c r="CN1" t="str">
+        <x:v>Владелец ПС</x:v>
+      </x:c>
+      <x:c r="CO1" t="str">
+        <x:v>pos-demo-owner</x:v>
+      </x:c>
+      <x:c r="CP1" t="str">
+        <x:v>Медианное время квалификации</x:v>
+      </x:c>
+      <x:c r="CQ1" t="str">
+        <x:v>metric-demo-duration</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="22.5" customHeight="1">
       <x:c r="A2" s="18" t="str">
@@ -22117,6 +22304,105 @@
       <x:c r="L2" s="18"/>
       <x:c r="M2" s="2"/>
       <x:c r="N2" s="2"/>
+      <x:c r="BA2" t="str">
+        <x:v>да</x:v>
+      </x:c>
+      <x:c r="BB2" t="str">
+        <x:v>применить</x:v>
+      </x:c>
+      <x:c r="BC2" t="str">
+        <x:v>принято</x:v>
+      </x:c>
+      <x:c r="BD2" t="str">
+        <x:v>текущая</x:v>
+      </x:c>
+      <x:c r="BE2" t="str">
+        <x:v>черновик</x:v>
+      </x:c>
+      <x:c r="BF2" t="str">
+        <x:v>исполняется</x:v>
+      </x:c>
+      <x:c r="BG2" t="str">
+        <x:v>человек</x:v>
+      </x:c>
+      <x:c r="BH2" t="str">
+        <x:v>активно</x:v>
+      </x:c>
+      <x:c r="BI2" t="str">
+        <x:v>организация</x:v>
+      </x:c>
+      <x:c r="BJ2" t="str">
+        <x:v>работа</x:v>
+      </x:c>
+      <x:c r="BK2" t="str">
+        <x:v>человек</x:v>
+      </x:c>
+      <x:c r="BL2" t="str">
+        <x:v>последовательность</x:v>
+      </x:c>
+      <x:c r="BM2" t="str">
+        <x:v>объект работы</x:v>
+      </x:c>
+      <x:c r="BN2" t="str">
+        <x:v>регламент</x:v>
+      </x:c>
+      <x:c r="BO2" t="str">
+        <x:v>проект</x:v>
+      </x:c>
+      <x:c r="BP2" t="str">
+        <x:v>входящая</x:v>
+      </x:c>
+      <x:c r="BQ2" t="str">
+        <x:v>за единицу</x:v>
+      </x:c>
+      <x:c r="BR2" t="str">
+        <x:v>создать</x:v>
+      </x:c>
+      <x:c r="BS2" t="str">
+        <x:v>карта бизнеса</x:v>
+      </x:c>
+      <x:c r="BT2" t="str">
+        <x:v>не готова</x:v>
+      </x:c>
+      <x:c r="BU2" t="str">
+        <x:v>разрешено</x:v>
+      </x:c>
+      <x:c r="BV2" t="str">
+        <x:v>критично</x:v>
+      </x:c>
+      <x:c r="BW2" t="str">
+        <x:v>действие</x:v>
+      </x:c>
+      <x:c r="BX2" t="str">
+        <x:v>кандидат</x:v>
+      </x:c>
+      <x:c r="BY2" t="str">
+        <x:v>инструментальное</x:v>
+      </x:c>
+      <x:c r="BZ2" t="str">
+        <x:v>интерфейс исполнения</x:v>
+      </x:c>
+      <x:c r="CA2" t="str">
+        <x:v>предполагается</x:v>
+      </x:c>
+      <x:c r="CB2" t="str">
+        <x:v>не проверено</x:v>
+      </x:c>
+      <x:c r="CC2" t="str">
+        <x:v>кандидат</x:v>
+      </x:c>
+      <x:c r="CD2" t="str">
+        <x:v>поддержана</x:v>
+      </x:c>
+      <x:c r="CE2" t="str">
+        <x:v>внедрить</x:v>
+      </x:c>
+      <x:c r="CF2" t="str">
+        <x:v>кандидат</x:v>
+      </x:c>
+      <x:c r="CG2" t="str">
+        <x:v>отклонение</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="28.5" customHeight="1">
       <x:c r="A3" s="21" t="str">
@@ -22135,6 +22421,105 @@
       <x:c r="L3" s="21"/>
       <x:c r="M3" s="2"/>
       <x:c r="N3" s="2"/>
+      <x:c r="BA3" t="str">
+        <x:v>нет</x:v>
+      </x:c>
+      <x:c r="BB3" t="str">
+        <x:v>исключить</x:v>
+      </x:c>
+      <x:c r="BC3" t="str">
+        <x:v>кандидат</x:v>
+      </x:c>
+      <x:c r="BD3" t="str">
+        <x:v>целевая</x:v>
+      </x:c>
+      <x:c r="BE3" t="str">
+        <x:v>принято</x:v>
+      </x:c>
+      <x:c r="BF3" t="str">
+        <x:v>не исполняется</x:v>
+      </x:c>
+      <x:c r="BG3" t="str">
+        <x:v>AI-агент</x:v>
+      </x:c>
+      <x:c r="BH3" t="str">
+        <x:v>завершено</x:v>
+      </x:c>
+      <x:c r="BI3" t="str">
+        <x:v>человек</x:v>
+      </x:c>
+      <x:c r="BJ3" t="str">
+        <x:v>решение</x:v>
+      </x:c>
+      <x:c r="BK3" t="str">
+        <x:v>AI-агент</x:v>
+      </x:c>
+      <x:c r="BL3" t="str">
+        <x:v>условие</x:v>
+      </x:c>
+      <x:c r="BM3" t="str">
+        <x:v>данные</x:v>
+      </x:c>
+      <x:c r="BN3" t="str">
+        <x:v>правило</x:v>
+      </x:c>
+      <x:c r="BO3" t="str">
+        <x:v>действует</x:v>
+      </x:c>
+      <x:c r="BP3" t="str">
+        <x:v>исходящая</x:v>
+      </x:c>
+      <x:c r="BQ3" t="str">
+        <x:v>фиксированная сумма</x:v>
+      </x:c>
+      <x:c r="BR3" t="str">
+        <x:v>изменить</x:v>
+      </x:c>
+      <x:c r="BS3" t="str">
+        <x:v>BPMN процесса</x:v>
+      </x:c>
+      <x:c r="BT3" t="str">
+        <x:v>готова к просмотру</x:v>
+      </x:c>
+      <x:c r="BU3" t="str">
+        <x:v>исключено</x:v>
+      </x:c>
+      <x:c r="BV3" t="str">
+        <x:v>предупреждение</x:v>
+      </x:c>
+      <x:c r="BW3" t="str">
+        <x:v>процесс</x:v>
+      </x:c>
+      <x:c r="BX3" t="str">
+        <x:v>подтверждено</x:v>
+      </x:c>
+      <x:c r="BY3" t="str">
+        <x:v>операционное</x:v>
+      </x:c>
+      <x:c r="BZ3" t="str">
+        <x:v>коммуникация</x:v>
+      </x:c>
+      <x:c r="CA3" t="str">
+        <x:v>подтверждена</x:v>
+      </x:c>
+      <x:c r="CB3" t="str">
+        <x:v>проверяется</x:v>
+      </x:c>
+      <x:c r="CC3" t="str">
+        <x:v>сформулирована</x:v>
+      </x:c>
+      <x:c r="CD3" t="str">
+        <x:v>опровергнута</x:v>
+      </x:c>
+      <x:c r="CE3" t="str">
+        <x:v>проверить ещё</x:v>
+      </x:c>
+      <x:c r="CF3" t="str">
+        <x:v>подготовлен</x:v>
+      </x:c>
+      <x:c r="CG3" t="str">
+        <x:v>гипотеза</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -22178,6 +22563,78 @@
       </x:c>
       <x:c r="N4" s="25" t="str">
         <x:v>notes</x:v>
+      </x:c>
+      <x:c r="BC4" t="str">
+        <x:v>гипотеза</x:v>
+      </x:c>
+      <x:c r="BE4" t="str">
+        <x:v>действует</x:v>
+      </x:c>
+      <x:c r="BF4" t="str">
+        <x:v>уточняется</x:v>
+      </x:c>
+      <x:c r="BH4" t="str">
+        <x:v>приостановлено</x:v>
+      </x:c>
+      <x:c r="BJ4" t="str">
+        <x:v>передача</x:v>
+      </x:c>
+      <x:c r="BK4" t="str">
+        <x:v>автоматизация</x:v>
+      </x:c>
+      <x:c r="BL4" t="str">
+        <x:v>ветвление</x:v>
+      </x:c>
+      <x:c r="BM4" t="str">
+        <x:v>вход</x:v>
+      </x:c>
+      <x:c r="BN4" t="str">
+        <x:v>данные</x:v>
+      </x:c>
+      <x:c r="BO4" t="str">
+        <x:v>приостановлен</x:v>
+      </x:c>
+      <x:c r="BQ4" t="str">
+        <x:v>подписка</x:v>
+      </x:c>
+      <x:c r="BR4" t="str">
+        <x:v>исключить</x:v>
+      </x:c>
+      <x:c r="BT4" t="str">
+        <x:v>готова к deployment</x:v>
+      </x:c>
+      <x:c r="BU4" t="str">
+        <x:v>ошибка</x:v>
+      </x:c>
+      <x:c r="BV4" t="str">
+        <x:v>информация</x:v>
+      </x:c>
+      <x:c r="BW4" t="str">
+        <x:v>производственная система</x:v>
+      </x:c>
+      <x:c r="BX4" t="str">
+        <x:v>в устранении</x:v>
+      </x:c>
+      <x:c r="BY4" t="str">
+        <x:v>системное</x:v>
+      </x:c>
+      <x:c r="CA4" t="str">
+        <x:v>не подтверждена</x:v>
+      </x:c>
+      <x:c r="CB4" t="str">
+        <x:v>подтверждено</x:v>
+      </x:c>
+      <x:c r="CC4" t="str">
+        <x:v>проверяется</x:v>
+      </x:c>
+      <x:c r="CD4" t="str">
+        <x:v>неопределённо</x:v>
+      </x:c>
+      <x:c r="CE4" t="str">
+        <x:v>отклонить</x:v>
+      </x:c>
+      <x:c r="CF4" t="str">
+        <x:v>разрешён</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
@@ -22195,6 +22652,57 @@
       <x:c r="L5" s="14"/>
       <x:c r="M5" s="14"/>
       <x:c r="N5" s="14"/>
+      <x:c r="BC5" t="str">
+        <x:v>конфликт</x:v>
+      </x:c>
+      <x:c r="BE5" t="str">
+        <x:v>закрыто</x:v>
+      </x:c>
+      <x:c r="BF5" t="str">
+        <x:v>не применимо</x:v>
+      </x:c>
+      <x:c r="BJ5" t="str">
+        <x:v>контроль</x:v>
+      </x:c>
+      <x:c r="BK5" t="str">
+        <x:v>совместно</x:v>
+      </x:c>
+      <x:c r="BL5" t="str">
+        <x:v>исключение</x:v>
+      </x:c>
+      <x:c r="BM5" t="str">
+        <x:v>выход</x:v>
+      </x:c>
+      <x:c r="BN5" t="str">
+        <x:v>источник истины</x:v>
+      </x:c>
+      <x:c r="BO5" t="str">
+        <x:v>закрыт</x:v>
+      </x:c>
+      <x:c r="BQ5" t="str">
+        <x:v>формула</x:v>
+      </x:c>
+      <x:c r="BR5" t="str">
+        <x:v>переход-версии</x:v>
+      </x:c>
+      <x:c r="BW5" t="str">
+        <x:v>объект</x:v>
+      </x:c>
+      <x:c r="BX5" t="str">
+        <x:v>проверяется</x:v>
+      </x:c>
+      <x:c r="BY5" t="str">
+        <x:v>не определено</x:v>
+      </x:c>
+      <x:c r="CB5" t="str">
+        <x:v>не подтверждено</x:v>
+      </x:c>
+      <x:c r="CC5" t="str">
+        <x:v>проверена</x:v>
+      </x:c>
+      <x:c r="CF5" t="str">
+        <x:v>выполняется</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="16.5" customHeight="1">
       <x:c r="A6" s="14"/>
@@ -22211,6 +22719,36 @@
       <x:c r="L6" s="14"/>
       <x:c r="M6" s="14"/>
       <x:c r="N6" s="14"/>
+      <x:c r="BC6" t="str">
+        <x:v>устарело</x:v>
+      </x:c>
+      <x:c r="BJ6" t="str">
+        <x:v>автоматизация</x:v>
+      </x:c>
+      <x:c r="BL6" t="str">
+        <x:v>возврат</x:v>
+      </x:c>
+      <x:c r="BM6" t="str">
+        <x:v>документ</x:v>
+      </x:c>
+      <x:c r="BN6" t="str">
+        <x:v>информационная система</x:v>
+      </x:c>
+      <x:c r="BR6" t="str">
+        <x:v>пересобрать-проекцию</x:v>
+      </x:c>
+      <x:c r="BW6" t="str">
+        <x:v>состояние</x:v>
+      </x:c>
+      <x:c r="BX6" t="str">
+        <x:v>закрыто</x:v>
+      </x:c>
+      <x:c r="CC6" t="str">
+        <x:v>закрыта</x:v>
+      </x:c>
+      <x:c r="CF6" t="str">
+        <x:v>завершён</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="16.5" customHeight="1">
       <x:c r="A7" s="14"/>
@@ -22227,6 +22765,27 @@
       <x:c r="L7" s="14"/>
       <x:c r="M7" s="14"/>
       <x:c r="N7" s="14"/>
+      <x:c r="BC7" t="str">
+        <x:v>неизвестно</x:v>
+      </x:c>
+      <x:c r="BJ7" t="str">
+        <x:v>подпроцесс</x:v>
+      </x:c>
+      <x:c r="BM7" t="str">
+        <x:v>ресурс</x:v>
+      </x:c>
+      <x:c r="BN7" t="str">
+        <x:v>интерфейс исполнения</x:v>
+      </x:c>
+      <x:c r="BW7" t="str">
+        <x:v>продукт</x:v>
+      </x:c>
+      <x:c r="BX7" t="str">
+        <x:v>не подтверждено</x:v>
+      </x:c>
+      <x:c r="CF7" t="str">
+        <x:v>остановлен</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="16.5" customHeight="1">
       <x:c r="A8" s="14"/>
@@ -22243,6 +22802,12 @@
       <x:c r="L8" s="14"/>
       <x:c r="M8" s="14"/>
       <x:c r="N8" s="14"/>
+      <x:c r="BN8" t="str">
+        <x:v>показатель</x:v>
+      </x:c>
+      <x:c r="BW8" t="str">
+        <x:v>материал</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="16.5" customHeight="1">
       <x:c r="A9" s="14"/>
@@ -22259,6 +22824,12 @@
       <x:c r="L9" s="14"/>
       <x:c r="M9" s="14"/>
       <x:c r="N9" s="14"/>
+      <x:c r="BN9" t="str">
+        <x:v>норматив</x:v>
+      </x:c>
+      <x:c r="BW9" t="str">
+        <x:v>показатель</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="16.5" customHeight="1">
       <x:c r="A10" s="14"/>
@@ -22275,6 +22846,9 @@
       <x:c r="L10" s="14"/>
       <x:c r="M10" s="14"/>
       <x:c r="N10" s="14"/>
+      <x:c r="BN10" t="str">
+        <x:v>SLA</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="16.5" customHeight="1">
       <x:c r="A11" s="14"/>
@@ -22291,6 +22865,9 @@
       <x:c r="L11" s="14"/>
       <x:c r="M11" s="14"/>
       <x:c r="N11" s="14"/>
+      <x:c r="BN11" t="str">
+        <x:v>автоматизация</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="16.5" customHeight="1">
       <x:c r="A12" s="14"/>
@@ -34054,9 +34631,15 @@
       </x:c>
       <x:c r="K5" s="28"/>
       <x:c r="L5" s="28"/>
-      <x:c r="M5" s="28"/>
-      <x:c r="N5" s="28"/>
-      <x:c r="O5" s="28"/>
+      <x:c r="M5" s="28" t="str">
+        <x:v>src-demo-regulation</x:v>
+      </x:c>
+      <x:c r="N5" s="28" t="str">
+        <x:v>Регламент обработки лидов</x:v>
+      </x:c>
+      <x:c r="O5" s="28" t="str">
+        <x:v>demo-regulation#sla</x:v>
+      </x:c>
       <x:c r="P5" s="28" t="str">
         <x:v>Лид обработан не позднее 3 дней</x:v>
       </x:c>
@@ -34085,12 +34668,20 @@
       <x:c r="AC5" s="28"/>
       <x:c r="AD5" s="28"/>
       <x:c r="AE5" s="28"/>
-      <x:c r="AF5" s="28"/>
-      <x:c r="AG5" s="28"/>
+      <x:c r="AF5" s="28" t="str">
+        <x:v>pos-demo-owner</x:v>
+      </x:c>
+      <x:c r="AG5" s="28" t="str">
+        <x:v>Владелец ПС</x:v>
+      </x:c>
       <x:c r="AH5" s="28"/>
       <x:c r="AI5" s="28"/>
-      <x:c r="AJ5" s="28"/>
-      <x:c r="AK5" s="28"/>
+      <x:c r="AJ5" s="28" t="str">
+        <x:v>dec-demo-deviation</x:v>
+      </x:c>
+      <x:c r="AK5" s="28" t="str">
+        <x:v>Подтвердить отклонение SLA</x:v>
+      </x:c>
       <x:c r="AL5" s="28"/>
       <x:c r="AM5" s="28"/>
       <x:c r="AN5" s="28" t="str">
@@ -37559,6 +38150,26 @@
     <x:mergeCell ref="A2:L2"/>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
+  <x:dataValidations count="6">
+    <x:dataValidation type="list" sqref="C5:C12">
+      <x:formula1>enum_deviation_status</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D5:D12">
+      <x:formula1>enum_deviation_type</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E5:E12">
+      <x:formula1>enum_development_scope_type</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="R5:R12">
+      <x:formula1>enum_evidence_channel</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AC5:AC12">
+      <x:formula1>enum_cause_status</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AH5:AH12">
+      <x:formula1>enum_verification_status</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -37575,16 +38186,16 @@
     <x:col min="6" max="6" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="19.440000534057617" hidden="0" customWidth="1"/>
@@ -37592,21 +38203,23 @@
     <x:col min="23" max="23" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="28" max="28" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="29" max="29" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="30" max="30" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="31" max="31" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="33" max="33" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="34" max="34" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="35" max="35" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="36" max="36" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="37" max="37" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="38" max="38" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="39" max="39" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="40" max="40" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="42" max="42" width="19.440000534057617" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
@@ -37652,6 +38265,8 @@
       <x:c r="AL1" s="2"/>
       <x:c r="AM1" s="2"/>
       <x:c r="AN1" s="2"/>
+      <x:c r="AO1" s="2"/>
+      <x:c r="AP1" s="2"/>
     </x:row>
     <x:row r="2" ht="22.5" customHeight="1">
       <x:c r="A2" s="18" t="str">
@@ -37696,6 +38311,8 @@
       <x:c r="AL2" s="2"/>
       <x:c r="AM2" s="2"/>
       <x:c r="AN2" s="2"/>
+      <x:c r="AO2" s="2"/>
+      <x:c r="AP2" s="2"/>
     </x:row>
     <x:row r="3" ht="28.5" customHeight="1">
       <x:c r="A3" s="21" t="str">
@@ -37740,6 +38357,8 @@
       <x:c r="AL3" s="2"/>
       <x:c r="AM3" s="2"/>
       <x:c r="AN3" s="2"/>
+      <x:c r="AO3" s="2"/>
+      <x:c r="AP3" s="2"/>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -37767,99 +38386,105 @@
         <x:v>new_opportunity</x:v>
       </x:c>
       <x:c r="I4" s="25" t="str">
+        <x:v>base_version_id</x:v>
+      </x:c>
+      <x:c r="J4" s="25" t="str">
+        <x:v>base_version_selector</x:v>
+      </x:c>
+      <x:c r="K4" s="25" t="str">
         <x:v>scope_type</x:v>
       </x:c>
-      <x:c r="J4" s="25" t="str">
+      <x:c r="L4" s="25" t="str">
         <x:v>scope_element_id</x:v>
       </x:c>
-      <x:c r="K4" s="25" t="str">
+      <x:c r="M4" s="25" t="str">
         <x:v>scope_element_selector</x:v>
       </x:c>
-      <x:c r="L4" s="25" t="str">
+      <x:c r="N4" s="25" t="str">
         <x:v>additional_impacts</x:v>
       </x:c>
-      <x:c r="M4" s="25" t="str">
+      <x:c r="O4" s="25" t="str">
         <x:v>proposed_change</x:v>
       </x:c>
-      <x:c r="N4" s="25" t="str">
+      <x:c r="P4" s="25" t="str">
         <x:v>mechanism</x:v>
       </x:c>
-      <x:c r="O4" s="25" t="str">
+      <x:c r="Q4" s="25" t="str">
         <x:v>primary_metric_id</x:v>
       </x:c>
-      <x:c r="P4" s="25" t="str">
+      <x:c r="R4" s="25" t="str">
         <x:v>primary_metric_selector</x:v>
       </x:c>
-      <x:c r="Q4" s="25" t="str">
+      <x:c r="S4" s="25" t="str">
         <x:v>baseline</x:v>
       </x:c>
-      <x:c r="R4" s="25" t="str">
+      <x:c r="T4" s="25" t="str">
         <x:v>expected_target</x:v>
       </x:c>
-      <x:c r="S4" s="25" t="str">
+      <x:c r="U4" s="25" t="str">
         <x:v>effect_horizon</x:v>
       </x:c>
-      <x:c r="T4" s="25" t="str">
+      <x:c r="V4" s="25" t="str">
         <x:v>support_criterion</x:v>
       </x:c>
-      <x:c r="U4" s="25" t="str">
+      <x:c r="W4" s="25" t="str">
         <x:v>refutation_criterion</x:v>
       </x:c>
-      <x:c r="V4" s="25" t="str">
+      <x:c r="X4" s="25" t="str">
         <x:v>inconclusive_criterion</x:v>
       </x:c>
-      <x:c r="W4" s="25" t="str">
+      <x:c r="Y4" s="25" t="str">
         <x:v>secondary_positive_effects</x:v>
       </x:c>
-      <x:c r="X4" s="25" t="str">
+      <x:c r="Z4" s="25" t="str">
         <x:v>secondary_negative_effects</x:v>
       </x:c>
-      <x:c r="Y4" s="25" t="str">
+      <x:c r="AA4" s="25" t="str">
         <x:v>soft_guardrails</x:v>
       </x:c>
-      <x:c r="Z4" s="25" t="str">
+      <x:c r="AB4" s="25" t="str">
         <x:v>responsible_position_id</x:v>
       </x:c>
-      <x:c r="AA4" s="25" t="str">
+      <x:c r="AC4" s="25" t="str">
         <x:v>responsible_position_selector</x:v>
       </x:c>
-      <x:c r="AB4" s="25" t="str">
+      <x:c r="AD4" s="25" t="str">
         <x:v>evidence_result</x:v>
       </x:c>
-      <x:c r="AC4" s="25" t="str">
+      <x:c r="AE4" s="25" t="str">
         <x:v>owner_decision</x:v>
       </x:c>
-      <x:c r="AD4" s="25" t="str">
+      <x:c r="AF4" s="25" t="str">
         <x:v>owner_decision_id</x:v>
       </x:c>
-      <x:c r="AE4" s="25" t="str">
+      <x:c r="AG4" s="25" t="str">
         <x:v>owner_decision_selector</x:v>
       </x:c>
-      <x:c r="AF4" s="25" t="str">
+      <x:c r="AH4" s="25" t="str">
         <x:v>resulting_version_id</x:v>
       </x:c>
-      <x:c r="AG4" s="25" t="str">
+      <x:c r="AI4" s="25" t="str">
         <x:v>resulting_version_selector</x:v>
       </x:c>
-      <x:c r="AH4" s="12" t="str">
+      <x:c r="AJ4" s="12" t="str">
         <x:v>next_step</x:v>
       </x:c>
-      <x:c r="AI4" s="25" t="str">
+      <x:c r="AK4" s="25" t="str">
         <x:v>due_date</x:v>
       </x:c>
-      <x:c r="AJ4" s="25" t="str">
+      <x:c r="AL4" s="25" t="str">
         <x:v>opened_at</x:v>
       </x:c>
-      <x:c r="AK4" s="25" t="str">
+      <x:c r="AM4" s="25" t="str">
         <x:v>formulated_at</x:v>
       </x:c>
-      <x:c r="AL4" s="25" t="str">
+      <x:c r="AN4" s="25" t="str">
         <x:v>tested_at</x:v>
       </x:c>
-      <x:c r="AM4" s="25" t="str">
+      <x:c r="AO4" s="25" t="str">
         <x:v>closed_at</x:v>
       </x:c>
-      <x:c r="AN4" s="25" t="str">
+      <x:c r="AP4" s="25" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -37889,55 +38514,77 @@
         <x:v>Разбирать звонок без ручного конспекта</x:v>
       </x:c>
       <x:c r="I5" s="28" t="str">
+        <x:v>ver-demo-v0.3</x:v>
+      </x:c>
+      <x:c r="J5" s="28" t="str">
+        <x:v>Текущая модель v0.3</x:v>
+      </x:c>
+      <x:c r="K5" s="28" t="str">
         <x:v>процесс</x:v>
       </x:c>
-      <x:c r="J5" s="28" t="str">
+      <x:c r="L5" s="28" t="str">
         <x:v>prc-demo-lead</x:v>
       </x:c>
-      <x:c r="K5" s="28" t="str">
+      <x:c r="M5" s="28" t="str">
         <x:v>Обработка лида</x:v>
       </x:c>
-      <x:c r="L5" s="28"/>
-      <x:c r="M5" s="28" t="str">
+      <x:c r="N5" s="28"/>
+      <x:c r="O5" s="28" t="str">
         <x:v>Добавить расшифровку после звонка</x:v>
       </x:c>
-      <x:c r="N5" s="28" t="str">
+      <x:c r="P5" s="28" t="str">
         <x:v>Менеджер меньше времени тратит на конспект</x:v>
       </x:c>
-      <x:c r="O5" s="28"/>
-      <x:c r="P5" s="28"/>
       <x:c r="Q5" s="28" t="str">
+        <x:v>metric-demo-duration</x:v>
+      </x:c>
+      <x:c r="R5" s="28" t="str">
+        <x:v>Медианное время квалификации</x:v>
+      </x:c>
+      <x:c r="S5" s="28" t="str">
         <x:v>20 минут</x:v>
       </x:c>
-      <x:c r="R5" s="28" t="str">
+      <x:c r="T5" s="28" t="str">
         <x:v>12 минут</x:v>
       </x:c>
-      <x:c r="S5" s="28"/>
-      <x:c r="T5" s="28"/>
-      <x:c r="U5" s="28"/>
-      <x:c r="V5" s="28"/>
-      <x:c r="W5" s="28"/>
-      <x:c r="X5" s="28"/>
+      <x:c r="U5" s="28" t="str">
+        <x:v>30 дней</x:v>
+      </x:c>
+      <x:c r="V5" s="28" t="str">
+        <x:v>Медиана не более 12 минут без снижения качества</x:v>
+      </x:c>
+      <x:c r="W5" s="28" t="str">
+        <x:v>Медиана не изменилась либо качество снизилось</x:v>
+      </x:c>
+      <x:c r="X5" s="28" t="str">
+        <x:v>Недостаточно наблюдений для вывода</x:v>
+      </x:c>
       <x:c r="Y5" s="28"/>
       <x:c r="Z5" s="28"/>
       <x:c r="AA5" s="28"/>
-      <x:c r="AB5" s="28"/>
-      <x:c r="AC5" s="28"/>
+      <x:c r="AB5" s="28" t="str">
+        <x:v>pos-demo-owner</x:v>
+      </x:c>
+      <x:c r="AC5" s="28" t="str">
+        <x:v>Владелец ПС</x:v>
+      </x:c>
       <x:c r="AD5" s="28"/>
       <x:c r="AE5" s="28"/>
       <x:c r="AF5" s="28"/>
       <x:c r="AG5" s="28"/>
-      <x:c r="AH5" s="28" t="str">
+      <x:c r="AH5" s="28"/>
+      <x:c r="AI5" s="28"/>
+      <x:c r="AJ5" s="28" t="str">
         <x:v>Подготовить эксперимент</x:v>
       </x:c>
-      <x:c r="AI5" s="30" t="n">
+      <x:c r="AK5" s="30" t="n">
         <x:v>46259</x:v>
       </x:c>
-      <x:c r="AJ5" s="29"/>
-      <x:c r="AK5" s="29"/>
       <x:c r="AL5" s="29"/>
       <x:c r="AM5" s="29"/>
-      <x:c r="AN5" s="28"/>
+      <x:c r="AN5" s="29"/>
+      <x:c r="AO5" s="29"/>
+      <x:c r="AP5" s="28"/>
     </x:row>
     <x:row r="6" ht="16.5" customHeight="1">
       <x:c r="A6" s="14"/>
@@ -37980,6 +38627,8 @@
       <x:c r="AL6" s="14"/>
       <x:c r="AM6" s="14"/>
       <x:c r="AN6" s="14"/>
+      <x:c r="AO6" s="14"/>
+      <x:c r="AP6" s="14"/>
     </x:row>
     <x:row r="7" ht="16.5" customHeight="1">
       <x:c r="A7" s="14"/>
@@ -38022,6 +38671,8 @@
       <x:c r="AL7" s="14"/>
       <x:c r="AM7" s="14"/>
       <x:c r="AN7" s="14"/>
+      <x:c r="AO7" s="14"/>
+      <x:c r="AP7" s="14"/>
     </x:row>
     <x:row r="8" ht="16.5" customHeight="1">
       <x:c r="A8" s="14"/>
@@ -38064,6 +38715,8 @@
       <x:c r="AL8" s="14"/>
       <x:c r="AM8" s="14"/>
       <x:c r="AN8" s="14"/>
+      <x:c r="AO8" s="14"/>
+      <x:c r="AP8" s="14"/>
     </x:row>
     <x:row r="9" ht="16.5" customHeight="1">
       <x:c r="A9" s="14"/>
@@ -38106,6 +38759,8 @@
       <x:c r="AL9" s="14"/>
       <x:c r="AM9" s="14"/>
       <x:c r="AN9" s="14"/>
+      <x:c r="AO9" s="14"/>
+      <x:c r="AP9" s="14"/>
     </x:row>
     <x:row r="10" ht="16.5" customHeight="1">
       <x:c r="A10" s="14"/>
@@ -38148,6 +38803,8 @@
       <x:c r="AL10" s="14"/>
       <x:c r="AM10" s="14"/>
       <x:c r="AN10" s="14"/>
+      <x:c r="AO10" s="14"/>
+      <x:c r="AP10" s="14"/>
     </x:row>
     <x:row r="11" ht="16.5" customHeight="1">
       <x:c r="A11" s="14"/>
@@ -38190,6 +38847,8 @@
       <x:c r="AL11" s="14"/>
       <x:c r="AM11" s="14"/>
       <x:c r="AN11" s="14"/>
+      <x:c r="AO11" s="14"/>
+      <x:c r="AP11" s="14"/>
     </x:row>
     <x:row r="12" ht="16.5" customHeight="1">
       <x:c r="A12" s="14"/>
@@ -38232,6 +38891,8 @@
       <x:c r="AL12" s="14"/>
       <x:c r="AM12" s="14"/>
       <x:c r="AN12" s="14"/>
+      <x:c r="AO12" s="14"/>
+      <x:c r="AP12" s="14"/>
     </x:row>
     <x:row r="13" ht="16.5" customHeight="1">
       <x:c r="A13" s="2"/>
@@ -38274,6 +38935,8 @@
       <x:c r="AL13" s="2"/>
       <x:c r="AM13" s="2"/>
       <x:c r="AN13" s="2"/>
+      <x:c r="AO13" s="2"/>
+      <x:c r="AP13" s="2"/>
     </x:row>
     <x:row r="14" ht="16.5" customHeight="1">
       <x:c r="A14" s="2"/>
@@ -38316,6 +38979,8 @@
       <x:c r="AL14" s="2"/>
       <x:c r="AM14" s="2"/>
       <x:c r="AN14" s="2"/>
+      <x:c r="AO14" s="2"/>
+      <x:c r="AP14" s="2"/>
     </x:row>
     <x:row r="15" ht="16.5" customHeight="1">
       <x:c r="A15" s="2"/>
@@ -38358,6 +39023,8 @@
       <x:c r="AL15" s="2"/>
       <x:c r="AM15" s="2"/>
       <x:c r="AN15" s="2"/>
+      <x:c r="AO15" s="2"/>
+      <x:c r="AP15" s="2"/>
     </x:row>
     <x:row r="16" ht="16.5" customHeight="1">
       <x:c r="A16" s="2"/>
@@ -38400,6 +39067,8 @@
       <x:c r="AL16" s="2"/>
       <x:c r="AM16" s="2"/>
       <x:c r="AN16" s="2"/>
+      <x:c r="AO16" s="2"/>
+      <x:c r="AP16" s="2"/>
     </x:row>
     <x:row r="17" ht="16.5" customHeight="1">
       <x:c r="A17" s="2"/>
@@ -38442,6 +39111,8 @@
       <x:c r="AL17" s="2"/>
       <x:c r="AM17" s="2"/>
       <x:c r="AN17" s="2"/>
+      <x:c r="AO17" s="2"/>
+      <x:c r="AP17" s="2"/>
     </x:row>
     <x:row r="18" ht="16.5" customHeight="1">
       <x:c r="A18" s="2"/>
@@ -38484,6 +39155,8 @@
       <x:c r="AL18" s="2"/>
       <x:c r="AM18" s="2"/>
       <x:c r="AN18" s="2"/>
+      <x:c r="AO18" s="2"/>
+      <x:c r="AP18" s="2"/>
     </x:row>
     <x:row r="19" ht="16.5" customHeight="1">
       <x:c r="A19" s="2"/>
@@ -38526,6 +39199,8 @@
       <x:c r="AL19" s="2"/>
       <x:c r="AM19" s="2"/>
       <x:c r="AN19" s="2"/>
+      <x:c r="AO19" s="2"/>
+      <x:c r="AP19" s="2"/>
     </x:row>
     <x:row r="20" ht="16.5" customHeight="1">
       <x:c r="A20" s="2"/>
@@ -38568,6 +39243,8 @@
       <x:c r="AL20" s="2"/>
       <x:c r="AM20" s="2"/>
       <x:c r="AN20" s="2"/>
+      <x:c r="AO20" s="2"/>
+      <x:c r="AP20" s="2"/>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
       <x:c r="A21" s="2"/>
@@ -38610,6 +39287,8 @@
       <x:c r="AL21" s="2"/>
       <x:c r="AM21" s="2"/>
       <x:c r="AN21" s="2"/>
+      <x:c r="AO21" s="2"/>
+      <x:c r="AP21" s="2"/>
     </x:row>
     <x:row r="22" ht="16.5" customHeight="1">
       <x:c r="A22" s="2"/>
@@ -38652,6 +39331,8 @@
       <x:c r="AL22" s="2"/>
       <x:c r="AM22" s="2"/>
       <x:c r="AN22" s="2"/>
+      <x:c r="AO22" s="2"/>
+      <x:c r="AP22" s="2"/>
     </x:row>
     <x:row r="23" ht="16.5" customHeight="1">
       <x:c r="A23" s="2"/>
@@ -38694,6 +39375,8 @@
       <x:c r="AL23" s="2"/>
       <x:c r="AM23" s="2"/>
       <x:c r="AN23" s="2"/>
+      <x:c r="AO23" s="2"/>
+      <x:c r="AP23" s="2"/>
     </x:row>
     <x:row r="24" ht="16.5" customHeight="1">
       <x:c r="A24" s="2"/>
@@ -38736,6 +39419,8 @@
       <x:c r="AL24" s="2"/>
       <x:c r="AM24" s="2"/>
       <x:c r="AN24" s="2"/>
+      <x:c r="AO24" s="2"/>
+      <x:c r="AP24" s="2"/>
     </x:row>
     <x:row r="25" ht="16.5" customHeight="1">
       <x:c r="A25" s="2"/>
@@ -38778,6 +39463,8 @@
       <x:c r="AL25" s="2"/>
       <x:c r="AM25" s="2"/>
       <x:c r="AN25" s="2"/>
+      <x:c r="AO25" s="2"/>
+      <x:c r="AP25" s="2"/>
     </x:row>
     <x:row r="26" ht="16.5" customHeight="1">
       <x:c r="A26" s="2"/>
@@ -38820,6 +39507,8 @@
       <x:c r="AL26" s="2"/>
       <x:c r="AM26" s="2"/>
       <x:c r="AN26" s="2"/>
+      <x:c r="AO26" s="2"/>
+      <x:c r="AP26" s="2"/>
     </x:row>
     <x:row r="27" ht="16.5" customHeight="1">
       <x:c r="A27" s="2"/>
@@ -38862,6 +39551,8 @@
       <x:c r="AL27" s="2"/>
       <x:c r="AM27" s="2"/>
       <x:c r="AN27" s="2"/>
+      <x:c r="AO27" s="2"/>
+      <x:c r="AP27" s="2"/>
     </x:row>
     <x:row r="28" ht="16.5" customHeight="1">
       <x:c r="A28" s="2"/>
@@ -38904,6 +39595,8 @@
       <x:c r="AL28" s="2"/>
       <x:c r="AM28" s="2"/>
       <x:c r="AN28" s="2"/>
+      <x:c r="AO28" s="2"/>
+      <x:c r="AP28" s="2"/>
     </x:row>
     <x:row r="29" ht="16.5" customHeight="1">
       <x:c r="A29" s="2"/>
@@ -38946,6 +39639,8 @@
       <x:c r="AL29" s="2"/>
       <x:c r="AM29" s="2"/>
       <x:c r="AN29" s="2"/>
+      <x:c r="AO29" s="2"/>
+      <x:c r="AP29" s="2"/>
     </x:row>
     <x:row r="30" ht="16.5" customHeight="1">
       <x:c r="A30" s="2"/>
@@ -38988,6 +39683,8 @@
       <x:c r="AL30" s="2"/>
       <x:c r="AM30" s="2"/>
       <x:c r="AN30" s="2"/>
+      <x:c r="AO30" s="2"/>
+      <x:c r="AP30" s="2"/>
     </x:row>
     <x:row r="31" ht="16.5" customHeight="1">
       <x:c r="A31" s="2"/>
@@ -39030,6 +39727,8 @@
       <x:c r="AL31" s="2"/>
       <x:c r="AM31" s="2"/>
       <x:c r="AN31" s="2"/>
+      <x:c r="AO31" s="2"/>
+      <x:c r="AP31" s="2"/>
     </x:row>
     <x:row r="32" ht="16.5" customHeight="1">
       <x:c r="A32" s="2"/>
@@ -39072,6 +39771,8 @@
       <x:c r="AL32" s="2"/>
       <x:c r="AM32" s="2"/>
       <x:c r="AN32" s="2"/>
+      <x:c r="AO32" s="2"/>
+      <x:c r="AP32" s="2"/>
     </x:row>
     <x:row r="33" ht="16.5" customHeight="1">
       <x:c r="A33" s="2"/>
@@ -39114,6 +39815,8 @@
       <x:c r="AL33" s="2"/>
       <x:c r="AM33" s="2"/>
       <x:c r="AN33" s="2"/>
+      <x:c r="AO33" s="2"/>
+      <x:c r="AP33" s="2"/>
     </x:row>
     <x:row r="34" ht="16.5" customHeight="1">
       <x:c r="A34" s="2"/>
@@ -39156,6 +39859,8 @@
       <x:c r="AL34" s="2"/>
       <x:c r="AM34" s="2"/>
       <x:c r="AN34" s="2"/>
+      <x:c r="AO34" s="2"/>
+      <x:c r="AP34" s="2"/>
     </x:row>
     <x:row r="35" ht="16.5" customHeight="1">
       <x:c r="A35" s="2"/>
@@ -39198,6 +39903,8 @@
       <x:c r="AL35" s="2"/>
       <x:c r="AM35" s="2"/>
       <x:c r="AN35" s="2"/>
+      <x:c r="AO35" s="2"/>
+      <x:c r="AP35" s="2"/>
     </x:row>
     <x:row r="36" ht="16.5" customHeight="1">
       <x:c r="A36" s="2"/>
@@ -39240,6 +39947,8 @@
       <x:c r="AL36" s="2"/>
       <x:c r="AM36" s="2"/>
       <x:c r="AN36" s="2"/>
+      <x:c r="AO36" s="2"/>
+      <x:c r="AP36" s="2"/>
     </x:row>
     <x:row r="37" ht="16.5" customHeight="1">
       <x:c r="A37" s="2"/>
@@ -39282,6 +39991,8 @@
       <x:c r="AL37" s="2"/>
       <x:c r="AM37" s="2"/>
       <x:c r="AN37" s="2"/>
+      <x:c r="AO37" s="2"/>
+      <x:c r="AP37" s="2"/>
     </x:row>
     <x:row r="38" ht="16.5" customHeight="1">
       <x:c r="A38" s="2"/>
@@ -39324,6 +40035,8 @@
       <x:c r="AL38" s="2"/>
       <x:c r="AM38" s="2"/>
       <x:c r="AN38" s="2"/>
+      <x:c r="AO38" s="2"/>
+      <x:c r="AP38" s="2"/>
     </x:row>
     <x:row r="39" ht="16.5" customHeight="1">
       <x:c r="A39" s="2"/>
@@ -39366,6 +40079,8 @@
       <x:c r="AL39" s="2"/>
       <x:c r="AM39" s="2"/>
       <x:c r="AN39" s="2"/>
+      <x:c r="AO39" s="2"/>
+      <x:c r="AP39" s="2"/>
     </x:row>
     <x:row r="40" ht="16.5" customHeight="1">
       <x:c r="A40" s="2"/>
@@ -39408,6 +40123,8 @@
       <x:c r="AL40" s="2"/>
       <x:c r="AM40" s="2"/>
       <x:c r="AN40" s="2"/>
+      <x:c r="AO40" s="2"/>
+      <x:c r="AP40" s="2"/>
     </x:row>
     <x:row r="41" ht="16.5" customHeight="1">
       <x:c r="A41" s="2"/>
@@ -39450,6 +40167,8 @@
       <x:c r="AL41" s="2"/>
       <x:c r="AM41" s="2"/>
       <x:c r="AN41" s="2"/>
+      <x:c r="AO41" s="2"/>
+      <x:c r="AP41" s="2"/>
     </x:row>
     <x:row r="42" ht="16.5" customHeight="1">
       <x:c r="A42" s="2"/>
@@ -39492,6 +40211,8 @@
       <x:c r="AL42" s="2"/>
       <x:c r="AM42" s="2"/>
       <x:c r="AN42" s="2"/>
+      <x:c r="AO42" s="2"/>
+      <x:c r="AP42" s="2"/>
     </x:row>
     <x:row r="43" ht="16.5" customHeight="1">
       <x:c r="A43" s="2"/>
@@ -39534,6 +40255,8 @@
       <x:c r="AL43" s="2"/>
       <x:c r="AM43" s="2"/>
       <x:c r="AN43" s="2"/>
+      <x:c r="AO43" s="2"/>
+      <x:c r="AP43" s="2"/>
     </x:row>
     <x:row r="44" ht="16.5" customHeight="1">
       <x:c r="A44" s="2"/>
@@ -39576,6 +40299,8 @@
       <x:c r="AL44" s="2"/>
       <x:c r="AM44" s="2"/>
       <x:c r="AN44" s="2"/>
+      <x:c r="AO44" s="2"/>
+      <x:c r="AP44" s="2"/>
     </x:row>
     <x:row r="45" ht="16.5" customHeight="1">
       <x:c r="A45" s="2"/>
@@ -39618,6 +40343,8 @@
       <x:c r="AL45" s="2"/>
       <x:c r="AM45" s="2"/>
       <x:c r="AN45" s="2"/>
+      <x:c r="AO45" s="2"/>
+      <x:c r="AP45" s="2"/>
     </x:row>
     <x:row r="46" ht="16.5" customHeight="1">
       <x:c r="A46" s="2"/>
@@ -39660,6 +40387,8 @@
       <x:c r="AL46" s="2"/>
       <x:c r="AM46" s="2"/>
       <x:c r="AN46" s="2"/>
+      <x:c r="AO46" s="2"/>
+      <x:c r="AP46" s="2"/>
     </x:row>
     <x:row r="47" ht="16.5" customHeight="1">
       <x:c r="A47" s="2"/>
@@ -39702,6 +40431,8 @@
       <x:c r="AL47" s="2"/>
       <x:c r="AM47" s="2"/>
       <x:c r="AN47" s="2"/>
+      <x:c r="AO47" s="2"/>
+      <x:c r="AP47" s="2"/>
     </x:row>
     <x:row r="48" ht="16.5" customHeight="1">
       <x:c r="A48" s="2"/>
@@ -39744,6 +40475,8 @@
       <x:c r="AL48" s="2"/>
       <x:c r="AM48" s="2"/>
       <x:c r="AN48" s="2"/>
+      <x:c r="AO48" s="2"/>
+      <x:c r="AP48" s="2"/>
     </x:row>
     <x:row r="49" ht="16.5" customHeight="1">
       <x:c r="A49" s="2"/>
@@ -39786,6 +40519,8 @@
       <x:c r="AL49" s="2"/>
       <x:c r="AM49" s="2"/>
       <x:c r="AN49" s="2"/>
+      <x:c r="AO49" s="2"/>
+      <x:c r="AP49" s="2"/>
     </x:row>
     <x:row r="50" ht="16.5" customHeight="1">
       <x:c r="A50" s="2"/>
@@ -39828,6 +40563,8 @@
       <x:c r="AL50" s="2"/>
       <x:c r="AM50" s="2"/>
       <x:c r="AN50" s="2"/>
+      <x:c r="AO50" s="2"/>
+      <x:c r="AP50" s="2"/>
     </x:row>
     <x:row r="51" ht="16.5" customHeight="1">
       <x:c r="A51" s="2"/>
@@ -39870,6 +40607,8 @@
       <x:c r="AL51" s="2"/>
       <x:c r="AM51" s="2"/>
       <x:c r="AN51" s="2"/>
+      <x:c r="AO51" s="2"/>
+      <x:c r="AP51" s="2"/>
     </x:row>
     <x:row r="52" ht="16.5" customHeight="1">
       <x:c r="A52" s="2"/>
@@ -39912,6 +40651,8 @@
       <x:c r="AL52" s="2"/>
       <x:c r="AM52" s="2"/>
       <x:c r="AN52" s="2"/>
+      <x:c r="AO52" s="2"/>
+      <x:c r="AP52" s="2"/>
     </x:row>
     <x:row r="53" ht="16.5" customHeight="1">
       <x:c r="A53" s="2"/>
@@ -39954,6 +40695,8 @@
       <x:c r="AL53" s="2"/>
       <x:c r="AM53" s="2"/>
       <x:c r="AN53" s="2"/>
+      <x:c r="AO53" s="2"/>
+      <x:c r="AP53" s="2"/>
     </x:row>
     <x:row r="54" ht="16.5" customHeight="1">
       <x:c r="A54" s="2"/>
@@ -39996,6 +40739,8 @@
       <x:c r="AL54" s="2"/>
       <x:c r="AM54" s="2"/>
       <x:c r="AN54" s="2"/>
+      <x:c r="AO54" s="2"/>
+      <x:c r="AP54" s="2"/>
     </x:row>
     <x:row r="55" ht="16.5" customHeight="1">
       <x:c r="A55" s="2"/>
@@ -40038,6 +40783,8 @@
       <x:c r="AL55" s="2"/>
       <x:c r="AM55" s="2"/>
       <x:c r="AN55" s="2"/>
+      <x:c r="AO55" s="2"/>
+      <x:c r="AP55" s="2"/>
     </x:row>
     <x:row r="56" ht="16.5" customHeight="1">
       <x:c r="A56" s="2"/>
@@ -40080,6 +40827,8 @@
       <x:c r="AL56" s="2"/>
       <x:c r="AM56" s="2"/>
       <x:c r="AN56" s="2"/>
+      <x:c r="AO56" s="2"/>
+      <x:c r="AP56" s="2"/>
     </x:row>
     <x:row r="57" ht="16.5" customHeight="1">
       <x:c r="A57" s="2"/>
@@ -40122,6 +40871,8 @@
       <x:c r="AL57" s="2"/>
       <x:c r="AM57" s="2"/>
       <x:c r="AN57" s="2"/>
+      <x:c r="AO57" s="2"/>
+      <x:c r="AP57" s="2"/>
     </x:row>
     <x:row r="58" ht="16.5" customHeight="1">
       <x:c r="A58" s="2"/>
@@ -40164,6 +40915,8 @@
       <x:c r="AL58" s="2"/>
       <x:c r="AM58" s="2"/>
       <x:c r="AN58" s="2"/>
+      <x:c r="AO58" s="2"/>
+      <x:c r="AP58" s="2"/>
     </x:row>
     <x:row r="59" ht="16.5" customHeight="1">
       <x:c r="A59" s="2"/>
@@ -40206,6 +40959,8 @@
       <x:c r="AL59" s="2"/>
       <x:c r="AM59" s="2"/>
       <x:c r="AN59" s="2"/>
+      <x:c r="AO59" s="2"/>
+      <x:c r="AP59" s="2"/>
     </x:row>
     <x:row r="60" ht="16.5" customHeight="1">
       <x:c r="A60" s="2"/>
@@ -40248,6 +41003,8 @@
       <x:c r="AL60" s="2"/>
       <x:c r="AM60" s="2"/>
       <x:c r="AN60" s="2"/>
+      <x:c r="AO60" s="2"/>
+      <x:c r="AP60" s="2"/>
     </x:row>
     <x:row r="61" ht="16.5" customHeight="1">
       <x:c r="A61" s="2"/>
@@ -40290,6 +41047,8 @@
       <x:c r="AL61" s="2"/>
       <x:c r="AM61" s="2"/>
       <x:c r="AN61" s="2"/>
+      <x:c r="AO61" s="2"/>
+      <x:c r="AP61" s="2"/>
     </x:row>
     <x:row r="62" ht="16.5" customHeight="1">
       <x:c r="A62" s="2"/>
@@ -40332,6 +41091,8 @@
       <x:c r="AL62" s="2"/>
       <x:c r="AM62" s="2"/>
       <x:c r="AN62" s="2"/>
+      <x:c r="AO62" s="2"/>
+      <x:c r="AP62" s="2"/>
     </x:row>
     <x:row r="63" ht="16.5" customHeight="1">
       <x:c r="A63" s="2"/>
@@ -40374,6 +41135,8 @@
       <x:c r="AL63" s="2"/>
       <x:c r="AM63" s="2"/>
       <x:c r="AN63" s="2"/>
+      <x:c r="AO63" s="2"/>
+      <x:c r="AP63" s="2"/>
     </x:row>
     <x:row r="64" ht="16.5" customHeight="1">
       <x:c r="A64" s="2"/>
@@ -40416,6 +41179,8 @@
       <x:c r="AL64" s="2"/>
       <x:c r="AM64" s="2"/>
       <x:c r="AN64" s="2"/>
+      <x:c r="AO64" s="2"/>
+      <x:c r="AP64" s="2"/>
     </x:row>
     <x:row r="65" ht="16.5" customHeight="1">
       <x:c r="A65" s="2"/>
@@ -40458,6 +41223,8 @@
       <x:c r="AL65" s="2"/>
       <x:c r="AM65" s="2"/>
       <x:c r="AN65" s="2"/>
+      <x:c r="AO65" s="2"/>
+      <x:c r="AP65" s="2"/>
     </x:row>
     <x:row r="66" ht="16.5" customHeight="1">
       <x:c r="A66" s="2"/>
@@ -40500,6 +41267,8 @@
       <x:c r="AL66" s="2"/>
       <x:c r="AM66" s="2"/>
       <x:c r="AN66" s="2"/>
+      <x:c r="AO66" s="2"/>
+      <x:c r="AP66" s="2"/>
     </x:row>
     <x:row r="67" ht="16.5" customHeight="1">
       <x:c r="A67" s="2"/>
@@ -40542,6 +41311,8 @@
       <x:c r="AL67" s="2"/>
       <x:c r="AM67" s="2"/>
       <x:c r="AN67" s="2"/>
+      <x:c r="AO67" s="2"/>
+      <x:c r="AP67" s="2"/>
     </x:row>
     <x:row r="68" ht="16.5" customHeight="1">
       <x:c r="A68" s="2"/>
@@ -40584,6 +41355,8 @@
       <x:c r="AL68" s="2"/>
       <x:c r="AM68" s="2"/>
       <x:c r="AN68" s="2"/>
+      <x:c r="AO68" s="2"/>
+      <x:c r="AP68" s="2"/>
     </x:row>
     <x:row r="69" ht="16.5" customHeight="1">
       <x:c r="A69" s="2"/>
@@ -40626,6 +41399,8 @@
       <x:c r="AL69" s="2"/>
       <x:c r="AM69" s="2"/>
       <x:c r="AN69" s="2"/>
+      <x:c r="AO69" s="2"/>
+      <x:c r="AP69" s="2"/>
     </x:row>
     <x:row r="70" ht="16.5" customHeight="1">
       <x:c r="A70" s="2"/>
@@ -40668,6 +41443,8 @@
       <x:c r="AL70" s="2"/>
       <x:c r="AM70" s="2"/>
       <x:c r="AN70" s="2"/>
+      <x:c r="AO70" s="2"/>
+      <x:c r="AP70" s="2"/>
     </x:row>
     <x:row r="71" ht="16.5" customHeight="1">
       <x:c r="A71" s="2"/>
@@ -40710,6 +41487,8 @@
       <x:c r="AL71" s="2"/>
       <x:c r="AM71" s="2"/>
       <x:c r="AN71" s="2"/>
+      <x:c r="AO71" s="2"/>
+      <x:c r="AP71" s="2"/>
     </x:row>
     <x:row r="72" ht="16.5" customHeight="1">
       <x:c r="A72" s="2"/>
@@ -40752,6 +41531,8 @@
       <x:c r="AL72" s="2"/>
       <x:c r="AM72" s="2"/>
       <x:c r="AN72" s="2"/>
+      <x:c r="AO72" s="2"/>
+      <x:c r="AP72" s="2"/>
     </x:row>
     <x:row r="73" ht="16.5" customHeight="1">
       <x:c r="A73" s="2"/>
@@ -40794,6 +41575,8 @@
       <x:c r="AL73" s="2"/>
       <x:c r="AM73" s="2"/>
       <x:c r="AN73" s="2"/>
+      <x:c r="AO73" s="2"/>
+      <x:c r="AP73" s="2"/>
     </x:row>
     <x:row r="74" ht="16.5" customHeight="1">
       <x:c r="A74" s="2"/>
@@ -40836,6 +41619,8 @@
       <x:c r="AL74" s="2"/>
       <x:c r="AM74" s="2"/>
       <x:c r="AN74" s="2"/>
+      <x:c r="AO74" s="2"/>
+      <x:c r="AP74" s="2"/>
     </x:row>
     <x:row r="75" ht="16.5" customHeight="1">
       <x:c r="A75" s="2"/>
@@ -40878,6 +41663,8 @@
       <x:c r="AL75" s="2"/>
       <x:c r="AM75" s="2"/>
       <x:c r="AN75" s="2"/>
+      <x:c r="AO75" s="2"/>
+      <x:c r="AP75" s="2"/>
     </x:row>
     <x:row r="76" ht="16.5" customHeight="1">
       <x:c r="A76" s="2"/>
@@ -40920,6 +41707,8 @@
       <x:c r="AL76" s="2"/>
       <x:c r="AM76" s="2"/>
       <x:c r="AN76" s="2"/>
+      <x:c r="AO76" s="2"/>
+      <x:c r="AP76" s="2"/>
     </x:row>
     <x:row r="77" ht="16.5" customHeight="1">
       <x:c r="A77" s="2"/>
@@ -40962,6 +41751,8 @@
       <x:c r="AL77" s="2"/>
       <x:c r="AM77" s="2"/>
       <x:c r="AN77" s="2"/>
+      <x:c r="AO77" s="2"/>
+      <x:c r="AP77" s="2"/>
     </x:row>
     <x:row r="78" ht="16.5" customHeight="1">
       <x:c r="A78" s="2"/>
@@ -41004,6 +41795,8 @@
       <x:c r="AL78" s="2"/>
       <x:c r="AM78" s="2"/>
       <x:c r="AN78" s="2"/>
+      <x:c r="AO78" s="2"/>
+      <x:c r="AP78" s="2"/>
     </x:row>
     <x:row r="79" ht="16.5" customHeight="1">
       <x:c r="A79" s="2"/>
@@ -41046,6 +41839,8 @@
       <x:c r="AL79" s="2"/>
       <x:c r="AM79" s="2"/>
       <x:c r="AN79" s="2"/>
+      <x:c r="AO79" s="2"/>
+      <x:c r="AP79" s="2"/>
     </x:row>
     <x:row r="80" ht="16.5" customHeight="1">
       <x:c r="A80" s="2"/>
@@ -41088,6 +41883,8 @@
       <x:c r="AL80" s="2"/>
       <x:c r="AM80" s="2"/>
       <x:c r="AN80" s="2"/>
+      <x:c r="AO80" s="2"/>
+      <x:c r="AP80" s="2"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -41095,6 +41892,20 @@
     <x:mergeCell ref="A2:L2"/>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
+  <x:dataValidations count="4">
+    <x:dataValidation type="list" sqref="C5:C12">
+      <x:formula1>enum_hypothesis_status</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K5:K12">
+      <x:formula1>enum_development_scope_type</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AD5:AD12">
+      <x:formula1>enum_evidence_result</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AE5:AE12">
+      <x:formula1>enum_development_decision</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -41466,6 +42277,7 @@
         <x:v>подготовлен</x:v>
       </x:c>
       <x:c r="D5" s="28" t="str">
+        <x:f>IF(A5="","",IF(AND(E5&lt;&gt;"",G5=""),"отклонение",IF(AND(E5="",G5&lt;&gt;""),"гипотеза","")))</x:f>
         <x:v>гипотеза</x:v>
       </x:c>
       <x:c r="E5" s="28"/>
@@ -41501,8 +42313,12 @@
       <x:c r="Q5" s="28" t="str">
         <x:v>Сравнить медианное время с baseline</x:v>
       </x:c>
-      <x:c r="R5" s="28"/>
-      <x:c r="S5" s="28"/>
+      <x:c r="R5" s="28" t="str">
+        <x:v>metric-demo-duration</x:v>
+      </x:c>
+      <x:c r="S5" s="28" t="str">
+        <x:v>Медианное время квалификации</x:v>
+      </x:c>
       <x:c r="T5" s="28" t="str">
         <x:v>20 минут</x:v>
       </x:c>
@@ -41511,12 +42327,20 @@
       </x:c>
       <x:c r="V5" s="28"/>
       <x:c r="W5" s="28"/>
-      <x:c r="X5" s="30"/>
-      <x:c r="Y5" s="30"/>
+      <x:c r="X5" s="30" t="n">
+        <x:v>46249</x:v>
+      </x:c>
+      <x:c r="Y5" s="30" t="n">
+        <x:v>46259</x:v>
+      </x:c>
       <x:c r="Z5" s="29"/>
       <x:c r="AA5" s="29"/>
-      <x:c r="AB5" s="28"/>
-      <x:c r="AC5" s="28"/>
+      <x:c r="AB5" s="28" t="str">
+        <x:v>pos-demo-owner</x:v>
+      </x:c>
+      <x:c r="AC5" s="28" t="str">
+        <x:v>Владелец ПС</x:v>
+      </x:c>
       <x:c r="AD5" s="28"/>
       <x:c r="AE5" s="28"/>
       <x:c r="AF5" s="28" t="str">
@@ -45301,6 +46125,23 @@
     <x:mergeCell ref="A2:L2"/>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
+  <x:dataValidations count="5">
+    <x:dataValidation type="list" sqref="C5:C12">
+      <x:formula1>enum_experiment_status</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D5:D12">
+      <x:formula1>enum_experiment_basis_type</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K5:K12">
+      <x:formula1>enum_development_scope_type</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AH5:AH12">
+      <x:formula1>enum_evidence_channel</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AO5:AO12">
+      <x:formula1>enum_development_decision</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -46484,15 +47325,27 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
-      <x:c r="A5" s="14"/>
-      <x:c r="B5" s="14"/>
-      <x:c r="C5" s="14"/>
-      <x:c r="D5" s="14"/>
+      <x:c r="A5" s="14" t="str">
+        <x:v>CHK-DEMO</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>демонстрация</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>предупреждение</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Review-XLSX содержит технические контракты</x:v>
+      </x:c>
       <x:c r="E5" s="14"/>
-      <x:c r="F5" s="14"/>
+      <x:c r="F5" s="14" t="str">
+        <x:v>OK</x:v>
+      </x:c>
       <x:c r="G5" s="14"/>
       <x:c r="H5" s="14"/>
-      <x:c r="I5" s="14"/>
+      <x:c r="I5" s="14" t="str">
+        <x:v>Каноническую проверку выполняет Google Sheets builder v0.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="16.5" customHeight="1">
       <x:c r="A6" s="14"/>
@@ -47325,6 +48178,11 @@
     <x:mergeCell ref="A2:I2"/>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="A5:I12">
+    <x:cfRule type="expression" dxfId="0" priority="1">
+      <x:formula>$F5="ERROR"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -50213,6 +51071,7 @@
         <x:v>selected_version_id</x:v>
       </x:c>
       <x:c r="E3" s="33" t="str">
+        <x:f>IF(B3="","",XLOOKUP(B3,selector_demo_versions,selector_demo_versions_ids,""))</x:f>
         <x:v>ver-demo-v0.3</x:v>
       </x:c>
       <x:c r="F3" s="2"/>
@@ -50262,6 +51121,7 @@
         <x:v>selected_system_id</x:v>
       </x:c>
       <x:c r="E4" s="33" t="str">
+        <x:f>IF(B4="","",XLOOKUP(B4,selector_demo_systems,selector_demo_systems_ids,""))</x:f>
         <x:v>ps-demo-attraction</x:v>
       </x:c>
       <x:c r="F4" s="2"/>
@@ -50311,6 +51171,7 @@
         <x:v>selected_process_id</x:v>
       </x:c>
       <x:c r="E5" s="33" t="str">
+        <x:f>IF(B5="","",XLOOKUP(B5,selector_demo_processes,selector_demo_processes_ids,""))</x:f>
         <x:v>prc-demo-lead</x:v>
       </x:c>
       <x:c r="F5" s="2"/>
@@ -53725,6 +54586,17 @@
     <x:mergeCell ref="A32:F32"/>
     <x:mergeCell ref="G32:L32"/>
   </x:mergeCells>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="B3">
+      <x:formula1>selector_demo_versions</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B4">
+      <x:formula1>selector_demo_systems</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B5">
+      <x:formula1>selector_demo_processes</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
fix: align v0.3 methodology and migration contracts
</commit_message>
<xml_diff>
--- a/outputs/v0.3-review/production-system-model-template-v0.3-review.xlsx
+++ b/outputs/v0.3-review/production-system-model-template-v0.3-review.xlsx
@@ -2,38 +2,38 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R0b3dca1709464630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Система" sheetId="2" r:id="Re60b5d214226498c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Схема шаблона" sheetId="3" r:id="R80280a7af63a4d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="4" r:id="Rb9187a0402fe439b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версии" sheetId="5" r:id="R7ca2923ced694aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исполнители" sheetId="6" r:id="R73e6818c8eb44a28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции" sheetId="7" r:id="Rbbe6743c120a4aad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Назначения" sheetId="8" r:id="R4c506565d622472f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контрагенты" sheetId="9" r:id="Re705a6aad1b54082"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Продукты" sheetId="10" r:id="R505d702d6be84e27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Материалы" sheetId="11" r:id="Rdd94ab43ccff4e45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процессы" sheetId="12" r:id="R0ff262c936e3422c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действия" sheetId="13" r:id="R3b39098b32004a22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи действий" sheetId="14" r:id="R62c6000634514408"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объекты" sheetId="15" r:id="R3a35579690bf4a6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Состояния" sheetId="16" r:id="R87f28f98d0eb4900"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переходы" sheetId="17" r:id="R511d0ff9eef24b6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Элементы модели" sheetId="18" r:id="R0dea83fddd074536"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контракты" sheetId="19" r:id="R986026adf49b4020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции контрактов" sheetId="20" r:id="Rcebfd67ffefa4517"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Интерфейсы передачи" sheetId="21" r:id="R239056d14fe743e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи модели" sheetId="22" r:id="Rcc64aaaba5e34cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Решения" sheetId="23" r:id="Rad6d7730ddb2452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения модели" sheetId="24" r:id="Rd7d8078d8e2148eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отклонения" sheetId="25" r:id="R3e09a0ff3486487f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гипотезы" sheetId="26" r:id="Rdebf444f9856493e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперименты" sheetId="27" r:id="Ra722a18f03424663"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез модели" sheetId="28" r:id="Rb1851d1b039c4976"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Проверки" sheetId="29" r:id="R4cbafd61b3aa4a9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр процессов" sheetId="30" r:id="R80f9f697e22f4c76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Рабочая панель" sheetId="31" r:id="R1ec4699c29e44e55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Диаграммы" sheetId="32" r:id="R53c3ac159ab243c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R83d98d95285f4652"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Система" sheetId="2" r:id="R16fd2f9b0a3446e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Схема шаблона" sheetId="3" r:id="Re5818f0deadd45ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="4" r:id="Rfba858c3fd364450"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версии" sheetId="5" r:id="R9d70a2599d6148ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исполнители" sheetId="6" r:id="R8951b197abb04acd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции" sheetId="7" r:id="Rb09807b6e16b43ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Назначения" sheetId="8" r:id="Rc998c3d6282f453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контрагенты" sheetId="9" r:id="R0dbcf0e2e2fd4a6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Продукты" sheetId="10" r:id="R09a3dd813b7e48a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Материалы" sheetId="11" r:id="R0741307f26234d77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процессы" sheetId="12" r:id="R65bf3039b10845ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действия" sheetId="13" r:id="R8b4382e373254675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи действий" sheetId="14" r:id="R56d696007720493c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объекты" sheetId="15" r:id="Raa6f64bb8d62445a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Состояния" sheetId="16" r:id="R497d067597784ed7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переходы" sheetId="17" r:id="R48200412d3104296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Элементы модели" sheetId="18" r:id="Rc81163db643f4c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контракты" sheetId="19" r:id="R05ef3011615b42d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции контрактов" sheetId="20" r:id="Rac4f35883ef646cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Интерфейсы передачи" sheetId="21" r:id="R948cfd217bd4434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи модели" sheetId="22" r:id="R689c2c12123d4bf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Решения" sheetId="23" r:id="R0fa9c976e6fb4cf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения модели" sheetId="24" r:id="R066a4760796345a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отклонения" sheetId="25" r:id="Rb2b5ecff5e004c7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гипотезы" sheetId="26" r:id="Rdeb43baaa5834cb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперименты" sheetId="27" r:id="Rf152118680944575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез модели" sheetId="28" r:id="Ra16cb255e9ff4245"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Проверки" sheetId="29" r:id="Rd5c0ac14d8ab49b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр процессов" sheetId="30" r:id="R1ef8fb0ed23948c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Рабочая панель" sheetId="31" r:id="Re5c398211e094101"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Диаграммы" sheetId="32" r:id="R191ac82d7c2544e9"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="enum_yes_no">'Система'!BA2:BA3</x:definedName>
@@ -48,7 +48,7 @@
     <x:definedName name="enum_action_type">'Система'!BJ2:BJ7</x:definedName>
     <x:definedName name="enum_performer_mode">'Система'!BK2:BK5</x:definedName>
     <x:definedName name="enum_edge_type">'Система'!BL2:BL6</x:definedName>
-    <x:definedName name="enum_object_type">'Система'!BM2:BM7</x:definedName>
+    <x:definedName name="enum_object_type">'Система'!BM2:BM5</x:definedName>
     <x:definedName name="enum_element_type">'Система'!BN2:BN11</x:definedName>
     <x:definedName name="enum_contract_status">'Система'!BO2:BO5</x:definedName>
     <x:definedName name="enum_direction">'Система'!BP2:BP3</x:definedName>
@@ -22565,7 +22565,7 @@
         <x:v>notes</x:v>
       </x:c>
       <x:c r="BC4" t="str">
-        <x:v>гипотеза</x:v>
+        <x:v>предположение</x:v>
       </x:c>
       <x:c r="BE4" t="str">
         <x:v>действует</x:v>
@@ -22586,7 +22586,7 @@
         <x:v>ветвление</x:v>
       </x:c>
       <x:c r="BM4" t="str">
-        <x:v>вход</x:v>
+        <x:v>документ</x:v>
       </x:c>
       <x:c r="BN4" t="str">
         <x:v>данные</x:v>
@@ -22671,7 +22671,7 @@
         <x:v>исключение</x:v>
       </x:c>
       <x:c r="BM5" t="str">
-        <x:v>выход</x:v>
+        <x:v>ресурс</x:v>
       </x:c>
       <x:c r="BN5" t="str">
         <x:v>источник истины</x:v>
@@ -22728,9 +22728,6 @@
       <x:c r="BL6" t="str">
         <x:v>возврат</x:v>
       </x:c>
-      <x:c r="BM6" t="str">
-        <x:v>документ</x:v>
-      </x:c>
       <x:c r="BN6" t="str">
         <x:v>информационная система</x:v>
       </x:c>
@@ -22770,9 +22767,6 @@
       </x:c>
       <x:c r="BJ7" t="str">
         <x:v>подпроцесс</x:v>
-      </x:c>
-      <x:c r="BM7" t="str">
-        <x:v>ресурс</x:v>
       </x:c>
       <x:c r="BN7" t="str">
         <x:v>интерфейс исполнения</x:v>
@@ -23997,21 +23991,23 @@
     <x:col min="8" max="8" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="19.440000534057617" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
@@ -24042,6 +24038,8 @@
       <x:c r="W1" s="2"/>
       <x:c r="X1" s="2"/>
       <x:c r="Y1" s="2"/>
+      <x:c r="Z1" s="2"/>
+      <x:c r="AA1" s="2"/>
     </x:row>
     <x:row r="2" ht="22.5" customHeight="1">
       <x:c r="A2" s="18" t="str">
@@ -24071,6 +24069,8 @@
       <x:c r="W2" s="2"/>
       <x:c r="X2" s="2"/>
       <x:c r="Y2" s="2"/>
+      <x:c r="Z2" s="2"/>
+      <x:c r="AA2" s="2"/>
     </x:row>
     <x:row r="3" ht="28.5" customHeight="1">
       <x:c r="A3" s="21" t="str">
@@ -24100,6 +24100,8 @@
       <x:c r="W3" s="2"/>
       <x:c r="X3" s="2"/>
       <x:c r="Y3" s="2"/>
+      <x:c r="Z3" s="2"/>
+      <x:c r="AA3" s="2"/>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -24120,61 +24122,67 @@
       <x:c r="F4" s="12" t="str">
         <x:v>direction</x:v>
       </x:c>
-      <x:c r="G4" s="12" t="str">
+      <x:c r="G4" s="25" t="str">
         <x:v>product_id</x:v>
       </x:c>
       <x:c r="H4" s="25" t="str">
         <x:v>product_selector</x:v>
       </x:c>
-      <x:c r="I4" s="12" t="str">
+      <x:c r="I4" s="25" t="str">
+        <x:v>material_id</x:v>
+      </x:c>
+      <x:c r="J4" s="25" t="str">
+        <x:v>material_selector</x:v>
+      </x:c>
+      <x:c r="K4" s="12" t="str">
         <x:v>internal_system_id</x:v>
       </x:c>
-      <x:c r="J4" s="25" t="str">
+      <x:c r="L4" s="25" t="str">
         <x:v>internal_system_selector</x:v>
       </x:c>
-      <x:c r="K4" s="12" t="str">
+      <x:c r="M4" s="12" t="str">
         <x:v>pricing_method</x:v>
       </x:c>
-      <x:c r="L4" s="25" t="str">
+      <x:c r="N4" s="25" t="str">
         <x:v>price_value</x:v>
       </x:c>
-      <x:c r="M4" s="25" t="str">
+      <x:c r="O4" s="25" t="str">
         <x:v>price_formula</x:v>
       </x:c>
-      <x:c r="N4" s="12" t="str">
+      <x:c r="P4" s="12" t="str">
         <x:v>currency</x:v>
       </x:c>
-      <x:c r="O4" s="12" t="str">
+      <x:c r="Q4" s="12" t="str">
         <x:v>pricing_unit</x:v>
       </x:c>
-      <x:c r="P4" s="25" t="str">
+      <x:c r="R4" s="25" t="str">
         <x:v>billing_trigger</x:v>
       </x:c>
-      <x:c r="Q4" s="25" t="str">
+      <x:c r="S4" s="25" t="str">
         <x:v>payment_terms</x:v>
       </x:c>
-      <x:c r="R4" s="25" t="str">
+      <x:c r="T4" s="25" t="str">
         <x:v>interface_id</x:v>
       </x:c>
-      <x:c r="S4" s="25" t="str">
+      <x:c r="U4" s="25" t="str">
         <x:v>interface_selector</x:v>
       </x:c>
-      <x:c r="T4" s="12" t="str">
+      <x:c r="V4" s="12" t="str">
         <x:v>knowledge_status</x:v>
       </x:c>
-      <x:c r="U4" s="12" t="str">
+      <x:c r="W4" s="12" t="str">
         <x:v>source_id</x:v>
       </x:c>
-      <x:c r="V4" s="25" t="str">
+      <x:c r="X4" s="25" t="str">
         <x:v>source_selector</x:v>
       </x:c>
-      <x:c r="W4" s="25" t="str">
+      <x:c r="Y4" s="25" t="str">
         <x:v>source_locator</x:v>
       </x:c>
-      <x:c r="X4" s="25" t="str">
+      <x:c r="Z4" s="25" t="str">
         <x:v>last_reviewed</x:v>
       </x:c>
-      <x:c r="Y4" s="25" t="str">
+      <x:c r="AA4" s="25" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -24204,6 +24212,8 @@
       <x:c r="W5" s="14"/>
       <x:c r="X5" s="14"/>
       <x:c r="Y5" s="14"/>
+      <x:c r="Z5" s="14"/>
+      <x:c r="AA5" s="14"/>
     </x:row>
     <x:row r="6" ht="16.5" customHeight="1">
       <x:c r="A6" s="14"/>
@@ -24231,6 +24241,8 @@
       <x:c r="W6" s="14"/>
       <x:c r="X6" s="14"/>
       <x:c r="Y6" s="14"/>
+      <x:c r="Z6" s="14"/>
+      <x:c r="AA6" s="14"/>
     </x:row>
     <x:row r="7" ht="16.5" customHeight="1">
       <x:c r="A7" s="14"/>
@@ -24258,6 +24270,8 @@
       <x:c r="W7" s="14"/>
       <x:c r="X7" s="14"/>
       <x:c r="Y7" s="14"/>
+      <x:c r="Z7" s="14"/>
+      <x:c r="AA7" s="14"/>
     </x:row>
     <x:row r="8" ht="16.5" customHeight="1">
       <x:c r="A8" s="14"/>
@@ -24285,6 +24299,8 @@
       <x:c r="W8" s="14"/>
       <x:c r="X8" s="14"/>
       <x:c r="Y8" s="14"/>
+      <x:c r="Z8" s="14"/>
+      <x:c r="AA8" s="14"/>
     </x:row>
     <x:row r="9" ht="16.5" customHeight="1">
       <x:c r="A9" s="14"/>
@@ -24312,6 +24328,8 @@
       <x:c r="W9" s="14"/>
       <x:c r="X9" s="14"/>
       <x:c r="Y9" s="14"/>
+      <x:c r="Z9" s="14"/>
+      <x:c r="AA9" s="14"/>
     </x:row>
     <x:row r="10" ht="16.5" customHeight="1">
       <x:c r="A10" s="14"/>
@@ -24339,6 +24357,8 @@
       <x:c r="W10" s="14"/>
       <x:c r="X10" s="14"/>
       <x:c r="Y10" s="14"/>
+      <x:c r="Z10" s="14"/>
+      <x:c r="AA10" s="14"/>
     </x:row>
     <x:row r="11" ht="16.5" customHeight="1">
       <x:c r="A11" s="14"/>
@@ -24366,6 +24386,8 @@
       <x:c r="W11" s="14"/>
       <x:c r="X11" s="14"/>
       <x:c r="Y11" s="14"/>
+      <x:c r="Z11" s="14"/>
+      <x:c r="AA11" s="14"/>
     </x:row>
     <x:row r="12" ht="16.5" customHeight="1">
       <x:c r="A12" s="14"/>
@@ -24393,6 +24415,8 @@
       <x:c r="W12" s="14"/>
       <x:c r="X12" s="14"/>
       <x:c r="Y12" s="14"/>
+      <x:c r="Z12" s="14"/>
+      <x:c r="AA12" s="14"/>
     </x:row>
     <x:row r="13" ht="16.5" customHeight="1">
       <x:c r="A13" s="2"/>
@@ -24420,6 +24444,8 @@
       <x:c r="W13" s="2"/>
       <x:c r="X13" s="2"/>
       <x:c r="Y13" s="2"/>
+      <x:c r="Z13" s="2"/>
+      <x:c r="AA13" s="2"/>
     </x:row>
     <x:row r="14" ht="16.5" customHeight="1">
       <x:c r="A14" s="2"/>
@@ -24447,6 +24473,8 @@
       <x:c r="W14" s="2"/>
       <x:c r="X14" s="2"/>
       <x:c r="Y14" s="2"/>
+      <x:c r="Z14" s="2"/>
+      <x:c r="AA14" s="2"/>
     </x:row>
     <x:row r="15" ht="16.5" customHeight="1">
       <x:c r="A15" s="2"/>
@@ -24474,6 +24502,8 @@
       <x:c r="W15" s="2"/>
       <x:c r="X15" s="2"/>
       <x:c r="Y15" s="2"/>
+      <x:c r="Z15" s="2"/>
+      <x:c r="AA15" s="2"/>
     </x:row>
     <x:row r="16" ht="16.5" customHeight="1">
       <x:c r="A16" s="2"/>
@@ -24501,6 +24531,8 @@
       <x:c r="W16" s="2"/>
       <x:c r="X16" s="2"/>
       <x:c r="Y16" s="2"/>
+      <x:c r="Z16" s="2"/>
+      <x:c r="AA16" s="2"/>
     </x:row>
     <x:row r="17" ht="16.5" customHeight="1">
       <x:c r="A17" s="2"/>
@@ -24528,6 +24560,8 @@
       <x:c r="W17" s="2"/>
       <x:c r="X17" s="2"/>
       <x:c r="Y17" s="2"/>
+      <x:c r="Z17" s="2"/>
+      <x:c r="AA17" s="2"/>
     </x:row>
     <x:row r="18" ht="16.5" customHeight="1">
       <x:c r="A18" s="2"/>
@@ -24555,6 +24589,8 @@
       <x:c r="W18" s="2"/>
       <x:c r="X18" s="2"/>
       <x:c r="Y18" s="2"/>
+      <x:c r="Z18" s="2"/>
+      <x:c r="AA18" s="2"/>
     </x:row>
     <x:row r="19" ht="16.5" customHeight="1">
       <x:c r="A19" s="2"/>
@@ -24582,6 +24618,8 @@
       <x:c r="W19" s="2"/>
       <x:c r="X19" s="2"/>
       <x:c r="Y19" s="2"/>
+      <x:c r="Z19" s="2"/>
+      <x:c r="AA19" s="2"/>
     </x:row>
     <x:row r="20" ht="16.5" customHeight="1">
       <x:c r="A20" s="2"/>
@@ -24609,6 +24647,8 @@
       <x:c r="W20" s="2"/>
       <x:c r="X20" s="2"/>
       <x:c r="Y20" s="2"/>
+      <x:c r="Z20" s="2"/>
+      <x:c r="AA20" s="2"/>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
       <x:c r="A21" s="2"/>
@@ -24636,6 +24676,8 @@
       <x:c r="W21" s="2"/>
       <x:c r="X21" s="2"/>
       <x:c r="Y21" s="2"/>
+      <x:c r="Z21" s="2"/>
+      <x:c r="AA21" s="2"/>
     </x:row>
     <x:row r="22" ht="16.5" customHeight="1">
       <x:c r="A22" s="2"/>
@@ -24663,6 +24705,8 @@
       <x:c r="W22" s="2"/>
       <x:c r="X22" s="2"/>
       <x:c r="Y22" s="2"/>
+      <x:c r="Z22" s="2"/>
+      <x:c r="AA22" s="2"/>
     </x:row>
     <x:row r="23" ht="16.5" customHeight="1">
       <x:c r="A23" s="2"/>
@@ -24690,6 +24734,8 @@
       <x:c r="W23" s="2"/>
       <x:c r="X23" s="2"/>
       <x:c r="Y23" s="2"/>
+      <x:c r="Z23" s="2"/>
+      <x:c r="AA23" s="2"/>
     </x:row>
     <x:row r="24" ht="16.5" customHeight="1">
       <x:c r="A24" s="2"/>
@@ -24717,6 +24763,8 @@
       <x:c r="W24" s="2"/>
       <x:c r="X24" s="2"/>
       <x:c r="Y24" s="2"/>
+      <x:c r="Z24" s="2"/>
+      <x:c r="AA24" s="2"/>
     </x:row>
     <x:row r="25" ht="16.5" customHeight="1">
       <x:c r="A25" s="2"/>
@@ -24744,6 +24792,8 @@
       <x:c r="W25" s="2"/>
       <x:c r="X25" s="2"/>
       <x:c r="Y25" s="2"/>
+      <x:c r="Z25" s="2"/>
+      <x:c r="AA25" s="2"/>
     </x:row>
     <x:row r="26" ht="16.5" customHeight="1">
       <x:c r="A26" s="2"/>
@@ -24771,6 +24821,8 @@
       <x:c r="W26" s="2"/>
       <x:c r="X26" s="2"/>
       <x:c r="Y26" s="2"/>
+      <x:c r="Z26" s="2"/>
+      <x:c r="AA26" s="2"/>
     </x:row>
     <x:row r="27" ht="16.5" customHeight="1">
       <x:c r="A27" s="2"/>
@@ -24798,6 +24850,8 @@
       <x:c r="W27" s="2"/>
       <x:c r="X27" s="2"/>
       <x:c r="Y27" s="2"/>
+      <x:c r="Z27" s="2"/>
+      <x:c r="AA27" s="2"/>
     </x:row>
     <x:row r="28" ht="16.5" customHeight="1">
       <x:c r="A28" s="2"/>
@@ -24825,6 +24879,8 @@
       <x:c r="W28" s="2"/>
       <x:c r="X28" s="2"/>
       <x:c r="Y28" s="2"/>
+      <x:c r="Z28" s="2"/>
+      <x:c r="AA28" s="2"/>
     </x:row>
     <x:row r="29" ht="16.5" customHeight="1">
       <x:c r="A29" s="2"/>
@@ -24852,6 +24908,8 @@
       <x:c r="W29" s="2"/>
       <x:c r="X29" s="2"/>
       <x:c r="Y29" s="2"/>
+      <x:c r="Z29" s="2"/>
+      <x:c r="AA29" s="2"/>
     </x:row>
     <x:row r="30" ht="16.5" customHeight="1">
       <x:c r="A30" s="2"/>
@@ -24879,6 +24937,8 @@
       <x:c r="W30" s="2"/>
       <x:c r="X30" s="2"/>
       <x:c r="Y30" s="2"/>
+      <x:c r="Z30" s="2"/>
+      <x:c r="AA30" s="2"/>
     </x:row>
     <x:row r="31" ht="16.5" customHeight="1">
       <x:c r="A31" s="2"/>
@@ -24906,6 +24966,8 @@
       <x:c r="W31" s="2"/>
       <x:c r="X31" s="2"/>
       <x:c r="Y31" s="2"/>
+      <x:c r="Z31" s="2"/>
+      <x:c r="AA31" s="2"/>
     </x:row>
     <x:row r="32" ht="16.5" customHeight="1">
       <x:c r="A32" s="2"/>
@@ -24933,6 +24995,8 @@
       <x:c r="W32" s="2"/>
       <x:c r="X32" s="2"/>
       <x:c r="Y32" s="2"/>
+      <x:c r="Z32" s="2"/>
+      <x:c r="AA32" s="2"/>
     </x:row>
     <x:row r="33" ht="16.5" customHeight="1">
       <x:c r="A33" s="2"/>
@@ -24960,6 +25024,8 @@
       <x:c r="W33" s="2"/>
       <x:c r="X33" s="2"/>
       <x:c r="Y33" s="2"/>
+      <x:c r="Z33" s="2"/>
+      <x:c r="AA33" s="2"/>
     </x:row>
     <x:row r="34" ht="16.5" customHeight="1">
       <x:c r="A34" s="2"/>
@@ -24987,6 +25053,8 @@
       <x:c r="W34" s="2"/>
       <x:c r="X34" s="2"/>
       <x:c r="Y34" s="2"/>
+      <x:c r="Z34" s="2"/>
+      <x:c r="AA34" s="2"/>
     </x:row>
     <x:row r="35" ht="16.5" customHeight="1">
       <x:c r="A35" s="2"/>
@@ -25014,6 +25082,8 @@
       <x:c r="W35" s="2"/>
       <x:c r="X35" s="2"/>
       <x:c r="Y35" s="2"/>
+      <x:c r="Z35" s="2"/>
+      <x:c r="AA35" s="2"/>
     </x:row>
     <x:row r="36" ht="16.5" customHeight="1">
       <x:c r="A36" s="2"/>
@@ -25041,6 +25111,8 @@
       <x:c r="W36" s="2"/>
       <x:c r="X36" s="2"/>
       <x:c r="Y36" s="2"/>
+      <x:c r="Z36" s="2"/>
+      <x:c r="AA36" s="2"/>
     </x:row>
     <x:row r="37" ht="16.5" customHeight="1">
       <x:c r="A37" s="2"/>
@@ -25068,6 +25140,8 @@
       <x:c r="W37" s="2"/>
       <x:c r="X37" s="2"/>
       <x:c r="Y37" s="2"/>
+      <x:c r="Z37" s="2"/>
+      <x:c r="AA37" s="2"/>
     </x:row>
     <x:row r="38" ht="16.5" customHeight="1">
       <x:c r="A38" s="2"/>
@@ -25095,6 +25169,8 @@
       <x:c r="W38" s="2"/>
       <x:c r="X38" s="2"/>
       <x:c r="Y38" s="2"/>
+      <x:c r="Z38" s="2"/>
+      <x:c r="AA38" s="2"/>
     </x:row>
     <x:row r="39" ht="16.5" customHeight="1">
       <x:c r="A39" s="2"/>
@@ -25122,6 +25198,8 @@
       <x:c r="W39" s="2"/>
       <x:c r="X39" s="2"/>
       <x:c r="Y39" s="2"/>
+      <x:c r="Z39" s="2"/>
+      <x:c r="AA39" s="2"/>
     </x:row>
     <x:row r="40" ht="16.5" customHeight="1">
       <x:c r="A40" s="2"/>
@@ -25149,6 +25227,8 @@
       <x:c r="W40" s="2"/>
       <x:c r="X40" s="2"/>
       <x:c r="Y40" s="2"/>
+      <x:c r="Z40" s="2"/>
+      <x:c r="AA40" s="2"/>
     </x:row>
     <x:row r="41" ht="16.5" customHeight="1">
       <x:c r="A41" s="2"/>
@@ -25176,6 +25256,8 @@
       <x:c r="W41" s="2"/>
       <x:c r="X41" s="2"/>
       <x:c r="Y41" s="2"/>
+      <x:c r="Z41" s="2"/>
+      <x:c r="AA41" s="2"/>
     </x:row>
     <x:row r="42" ht="16.5" customHeight="1">
       <x:c r="A42" s="2"/>
@@ -25203,6 +25285,8 @@
       <x:c r="W42" s="2"/>
       <x:c r="X42" s="2"/>
       <x:c r="Y42" s="2"/>
+      <x:c r="Z42" s="2"/>
+      <x:c r="AA42" s="2"/>
     </x:row>
     <x:row r="43" ht="16.5" customHeight="1">
       <x:c r="A43" s="2"/>
@@ -25230,6 +25314,8 @@
       <x:c r="W43" s="2"/>
       <x:c r="X43" s="2"/>
       <x:c r="Y43" s="2"/>
+      <x:c r="Z43" s="2"/>
+      <x:c r="AA43" s="2"/>
     </x:row>
     <x:row r="44" ht="16.5" customHeight="1">
       <x:c r="A44" s="2"/>
@@ -25257,6 +25343,8 @@
       <x:c r="W44" s="2"/>
       <x:c r="X44" s="2"/>
       <x:c r="Y44" s="2"/>
+      <x:c r="Z44" s="2"/>
+      <x:c r="AA44" s="2"/>
     </x:row>
     <x:row r="45" ht="16.5" customHeight="1">
       <x:c r="A45" s="2"/>
@@ -25284,6 +25372,8 @@
       <x:c r="W45" s="2"/>
       <x:c r="X45" s="2"/>
       <x:c r="Y45" s="2"/>
+      <x:c r="Z45" s="2"/>
+      <x:c r="AA45" s="2"/>
     </x:row>
     <x:row r="46" ht="16.5" customHeight="1">
       <x:c r="A46" s="2"/>
@@ -25311,6 +25401,8 @@
       <x:c r="W46" s="2"/>
       <x:c r="X46" s="2"/>
       <x:c r="Y46" s="2"/>
+      <x:c r="Z46" s="2"/>
+      <x:c r="AA46" s="2"/>
     </x:row>
     <x:row r="47" ht="16.5" customHeight="1">
       <x:c r="A47" s="2"/>
@@ -25338,6 +25430,8 @@
       <x:c r="W47" s="2"/>
       <x:c r="X47" s="2"/>
       <x:c r="Y47" s="2"/>
+      <x:c r="Z47" s="2"/>
+      <x:c r="AA47" s="2"/>
     </x:row>
     <x:row r="48" ht="16.5" customHeight="1">
       <x:c r="A48" s="2"/>
@@ -25365,6 +25459,8 @@
       <x:c r="W48" s="2"/>
       <x:c r="X48" s="2"/>
       <x:c r="Y48" s="2"/>
+      <x:c r="Z48" s="2"/>
+      <x:c r="AA48" s="2"/>
     </x:row>
     <x:row r="49" ht="16.5" customHeight="1">
       <x:c r="A49" s="2"/>
@@ -25392,6 +25488,8 @@
       <x:c r="W49" s="2"/>
       <x:c r="X49" s="2"/>
       <x:c r="Y49" s="2"/>
+      <x:c r="Z49" s="2"/>
+      <x:c r="AA49" s="2"/>
     </x:row>
     <x:row r="50" ht="16.5" customHeight="1">
       <x:c r="A50" s="2"/>
@@ -25419,6 +25517,8 @@
       <x:c r="W50" s="2"/>
       <x:c r="X50" s="2"/>
       <x:c r="Y50" s="2"/>
+      <x:c r="Z50" s="2"/>
+      <x:c r="AA50" s="2"/>
     </x:row>
     <x:row r="51" ht="16.5" customHeight="1">
       <x:c r="A51" s="2"/>
@@ -25446,6 +25546,8 @@
       <x:c r="W51" s="2"/>
       <x:c r="X51" s="2"/>
       <x:c r="Y51" s="2"/>
+      <x:c r="Z51" s="2"/>
+      <x:c r="AA51" s="2"/>
     </x:row>
     <x:row r="52" ht="16.5" customHeight="1">
       <x:c r="A52" s="2"/>
@@ -25473,6 +25575,8 @@
       <x:c r="W52" s="2"/>
       <x:c r="X52" s="2"/>
       <x:c r="Y52" s="2"/>
+      <x:c r="Z52" s="2"/>
+      <x:c r="AA52" s="2"/>
     </x:row>
     <x:row r="53" ht="16.5" customHeight="1">
       <x:c r="A53" s="2"/>
@@ -25500,6 +25604,8 @@
       <x:c r="W53" s="2"/>
       <x:c r="X53" s="2"/>
       <x:c r="Y53" s="2"/>
+      <x:c r="Z53" s="2"/>
+      <x:c r="AA53" s="2"/>
     </x:row>
     <x:row r="54" ht="16.5" customHeight="1">
       <x:c r="A54" s="2"/>
@@ -25527,6 +25633,8 @@
       <x:c r="W54" s="2"/>
       <x:c r="X54" s="2"/>
       <x:c r="Y54" s="2"/>
+      <x:c r="Z54" s="2"/>
+      <x:c r="AA54" s="2"/>
     </x:row>
     <x:row r="55" ht="16.5" customHeight="1">
       <x:c r="A55" s="2"/>
@@ -25554,6 +25662,8 @@
       <x:c r="W55" s="2"/>
       <x:c r="X55" s="2"/>
       <x:c r="Y55" s="2"/>
+      <x:c r="Z55" s="2"/>
+      <x:c r="AA55" s="2"/>
     </x:row>
     <x:row r="56" ht="16.5" customHeight="1">
       <x:c r="A56" s="2"/>
@@ -25581,6 +25691,8 @@
       <x:c r="W56" s="2"/>
       <x:c r="X56" s="2"/>
       <x:c r="Y56" s="2"/>
+      <x:c r="Z56" s="2"/>
+      <x:c r="AA56" s="2"/>
     </x:row>
     <x:row r="57" ht="16.5" customHeight="1">
       <x:c r="A57" s="2"/>
@@ -25608,6 +25720,8 @@
       <x:c r="W57" s="2"/>
       <x:c r="X57" s="2"/>
       <x:c r="Y57" s="2"/>
+      <x:c r="Z57" s="2"/>
+      <x:c r="AA57" s="2"/>
     </x:row>
     <x:row r="58" ht="16.5" customHeight="1">
       <x:c r="A58" s="2"/>
@@ -25635,6 +25749,8 @@
       <x:c r="W58" s="2"/>
       <x:c r="X58" s="2"/>
       <x:c r="Y58" s="2"/>
+      <x:c r="Z58" s="2"/>
+      <x:c r="AA58" s="2"/>
     </x:row>
     <x:row r="59" ht="16.5" customHeight="1">
       <x:c r="A59" s="2"/>
@@ -25662,6 +25778,8 @@
       <x:c r="W59" s="2"/>
       <x:c r="X59" s="2"/>
       <x:c r="Y59" s="2"/>
+      <x:c r="Z59" s="2"/>
+      <x:c r="AA59" s="2"/>
     </x:row>
     <x:row r="60" ht="16.5" customHeight="1">
       <x:c r="A60" s="2"/>
@@ -25689,6 +25807,8 @@
       <x:c r="W60" s="2"/>
       <x:c r="X60" s="2"/>
       <x:c r="Y60" s="2"/>
+      <x:c r="Z60" s="2"/>
+      <x:c r="AA60" s="2"/>
     </x:row>
     <x:row r="61" ht="16.5" customHeight="1">
       <x:c r="A61" s="2"/>
@@ -25716,6 +25836,8 @@
       <x:c r="W61" s="2"/>
       <x:c r="X61" s="2"/>
       <x:c r="Y61" s="2"/>
+      <x:c r="Z61" s="2"/>
+      <x:c r="AA61" s="2"/>
     </x:row>
     <x:row r="62" ht="16.5" customHeight="1">
       <x:c r="A62" s="2"/>
@@ -25743,6 +25865,8 @@
       <x:c r="W62" s="2"/>
       <x:c r="X62" s="2"/>
       <x:c r="Y62" s="2"/>
+      <x:c r="Z62" s="2"/>
+      <x:c r="AA62" s="2"/>
     </x:row>
     <x:row r="63" ht="16.5" customHeight="1">
       <x:c r="A63" s="2"/>
@@ -25770,6 +25894,8 @@
       <x:c r="W63" s="2"/>
       <x:c r="X63" s="2"/>
       <x:c r="Y63" s="2"/>
+      <x:c r="Z63" s="2"/>
+      <x:c r="AA63" s="2"/>
     </x:row>
     <x:row r="64" ht="16.5" customHeight="1">
       <x:c r="A64" s="2"/>
@@ -25797,6 +25923,8 @@
       <x:c r="W64" s="2"/>
       <x:c r="X64" s="2"/>
       <x:c r="Y64" s="2"/>
+      <x:c r="Z64" s="2"/>
+      <x:c r="AA64" s="2"/>
     </x:row>
     <x:row r="65" ht="16.5" customHeight="1">
       <x:c r="A65" s="2"/>
@@ -25824,6 +25952,8 @@
       <x:c r="W65" s="2"/>
       <x:c r="X65" s="2"/>
       <x:c r="Y65" s="2"/>
+      <x:c r="Z65" s="2"/>
+      <x:c r="AA65" s="2"/>
     </x:row>
     <x:row r="66" ht="16.5" customHeight="1">
       <x:c r="A66" s="2"/>
@@ -25851,6 +25981,8 @@
       <x:c r="W66" s="2"/>
       <x:c r="X66" s="2"/>
       <x:c r="Y66" s="2"/>
+      <x:c r="Z66" s="2"/>
+      <x:c r="AA66" s="2"/>
     </x:row>
     <x:row r="67" ht="16.5" customHeight="1">
       <x:c r="A67" s="2"/>
@@ -25878,6 +26010,8 @@
       <x:c r="W67" s="2"/>
       <x:c r="X67" s="2"/>
       <x:c r="Y67" s="2"/>
+      <x:c r="Z67" s="2"/>
+      <x:c r="AA67" s="2"/>
     </x:row>
     <x:row r="68" ht="16.5" customHeight="1">
       <x:c r="A68" s="2"/>
@@ -25905,6 +26039,8 @@
       <x:c r="W68" s="2"/>
       <x:c r="X68" s="2"/>
       <x:c r="Y68" s="2"/>
+      <x:c r="Z68" s="2"/>
+      <x:c r="AA68" s="2"/>
     </x:row>
     <x:row r="69" ht="16.5" customHeight="1">
       <x:c r="A69" s="2"/>
@@ -25932,6 +26068,8 @@
       <x:c r="W69" s="2"/>
       <x:c r="X69" s="2"/>
       <x:c r="Y69" s="2"/>
+      <x:c r="Z69" s="2"/>
+      <x:c r="AA69" s="2"/>
     </x:row>
     <x:row r="70" ht="16.5" customHeight="1">
       <x:c r="A70" s="2"/>
@@ -25959,6 +26097,8 @@
       <x:c r="W70" s="2"/>
       <x:c r="X70" s="2"/>
       <x:c r="Y70" s="2"/>
+      <x:c r="Z70" s="2"/>
+      <x:c r="AA70" s="2"/>
     </x:row>
     <x:row r="71" ht="16.5" customHeight="1">
       <x:c r="A71" s="2"/>
@@ -25986,6 +26126,8 @@
       <x:c r="W71" s="2"/>
       <x:c r="X71" s="2"/>
       <x:c r="Y71" s="2"/>
+      <x:c r="Z71" s="2"/>
+      <x:c r="AA71" s="2"/>
     </x:row>
     <x:row r="72" ht="16.5" customHeight="1">
       <x:c r="A72" s="2"/>
@@ -26013,6 +26155,8 @@
       <x:c r="W72" s="2"/>
       <x:c r="X72" s="2"/>
       <x:c r="Y72" s="2"/>
+      <x:c r="Z72" s="2"/>
+      <x:c r="AA72" s="2"/>
     </x:row>
     <x:row r="73" ht="16.5" customHeight="1">
       <x:c r="A73" s="2"/>
@@ -26040,6 +26184,8 @@
       <x:c r="W73" s="2"/>
       <x:c r="X73" s="2"/>
       <x:c r="Y73" s="2"/>
+      <x:c r="Z73" s="2"/>
+      <x:c r="AA73" s="2"/>
     </x:row>
     <x:row r="74" ht="16.5" customHeight="1">
       <x:c r="A74" s="2"/>
@@ -26067,6 +26213,8 @@
       <x:c r="W74" s="2"/>
       <x:c r="X74" s="2"/>
       <x:c r="Y74" s="2"/>
+      <x:c r="Z74" s="2"/>
+      <x:c r="AA74" s="2"/>
     </x:row>
     <x:row r="75" ht="16.5" customHeight="1">
       <x:c r="A75" s="2"/>
@@ -26094,6 +26242,8 @@
       <x:c r="W75" s="2"/>
       <x:c r="X75" s="2"/>
       <x:c r="Y75" s="2"/>
+      <x:c r="Z75" s="2"/>
+      <x:c r="AA75" s="2"/>
     </x:row>
     <x:row r="76" ht="16.5" customHeight="1">
       <x:c r="A76" s="2"/>
@@ -26121,6 +26271,8 @@
       <x:c r="W76" s="2"/>
       <x:c r="X76" s="2"/>
       <x:c r="Y76" s="2"/>
+      <x:c r="Z76" s="2"/>
+      <x:c r="AA76" s="2"/>
     </x:row>
     <x:row r="77" ht="16.5" customHeight="1">
       <x:c r="A77" s="2"/>
@@ -26148,6 +26300,8 @@
       <x:c r="W77" s="2"/>
       <x:c r="X77" s="2"/>
       <x:c r="Y77" s="2"/>
+      <x:c r="Z77" s="2"/>
+      <x:c r="AA77" s="2"/>
     </x:row>
     <x:row r="78" ht="16.5" customHeight="1">
       <x:c r="A78" s="2"/>
@@ -26175,6 +26329,8 @@
       <x:c r="W78" s="2"/>
       <x:c r="X78" s="2"/>
       <x:c r="Y78" s="2"/>
+      <x:c r="Z78" s="2"/>
+      <x:c r="AA78" s="2"/>
     </x:row>
     <x:row r="79" ht="16.5" customHeight="1">
       <x:c r="A79" s="2"/>
@@ -26202,6 +26358,8 @@
       <x:c r="W79" s="2"/>
       <x:c r="X79" s="2"/>
       <x:c r="Y79" s="2"/>
+      <x:c r="Z79" s="2"/>
+      <x:c r="AA79" s="2"/>
     </x:row>
     <x:row r="80" ht="16.5" customHeight="1">
       <x:c r="A80" s="2"/>
@@ -26229,6 +26387,8 @@
       <x:c r="W80" s="2"/>
       <x:c r="X80" s="2"/>
       <x:c r="Y80" s="2"/>
+      <x:c r="Z80" s="2"/>
+      <x:c r="AA80" s="2"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -26254,24 +26414,26 @@
     <x:col min="8" max="8" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="19.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="16.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="26.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="19.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="27" max="27" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="16.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="26.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="19.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="19.440000534057617" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
@@ -26305,6 +26467,8 @@
       <x:c r="Z1" s="2"/>
       <x:c r="AA1" s="2"/>
       <x:c r="AB1" s="2"/>
+      <x:c r="AC1" s="2"/>
+      <x:c r="AD1" s="2"/>
     </x:row>
     <x:row r="2" ht="22.5" customHeight="1">
       <x:c r="A2" s="18" t="str">
@@ -26337,6 +26501,8 @@
       <x:c r="Z2" s="2"/>
       <x:c r="AA2" s="2"/>
       <x:c r="AB2" s="2"/>
+      <x:c r="AC2" s="2"/>
+      <x:c r="AD2" s="2"/>
     </x:row>
     <x:row r="3" ht="28.5" customHeight="1">
       <x:c r="A3" s="21" t="str">
@@ -26369,6 +26535,8 @@
       <x:c r="Z3" s="2"/>
       <x:c r="AA3" s="2"/>
       <x:c r="AB3" s="2"/>
+      <x:c r="AC3" s="2"/>
+      <x:c r="AD3" s="2"/>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -26395,64 +26563,70 @@
       <x:c r="H4" s="25" t="str">
         <x:v>internal_system_selector</x:v>
       </x:c>
-      <x:c r="I4" s="12" t="str">
+      <x:c r="I4" s="25" t="str">
         <x:v>product_id</x:v>
       </x:c>
       <x:c r="J4" s="25" t="str">
         <x:v>product_selector</x:v>
       </x:c>
-      <x:c r="K4" s="12" t="str">
+      <x:c r="K4" s="25" t="str">
+        <x:v>material_id</x:v>
+      </x:c>
+      <x:c r="L4" s="25" t="str">
+        <x:v>material_selector</x:v>
+      </x:c>
+      <x:c r="M4" s="12" t="str">
         <x:v>transfer_trigger</x:v>
       </x:c>
-      <x:c r="L4" s="12" t="str">
+      <x:c r="N4" s="12" t="str">
         <x:v>channel</x:v>
       </x:c>
-      <x:c r="M4" s="25" t="str">
+      <x:c r="O4" s="25" t="str">
         <x:v>information_system_id</x:v>
       </x:c>
-      <x:c r="N4" s="25" t="str">
+      <x:c r="P4" s="25" t="str">
         <x:v>information_system_selector</x:v>
       </x:c>
-      <x:c r="O4" s="12" t="str">
+      <x:c r="Q4" s="12" t="str">
         <x:v>format_description</x:v>
       </x:c>
-      <x:c r="P4" s="25" t="str">
+      <x:c r="R4" s="25" t="str">
         <x:v>package_description</x:v>
       </x:c>
-      <x:c r="Q4" s="25" t="str">
+      <x:c r="S4" s="25" t="str">
         <x:v>acceptance_action_id</x:v>
       </x:c>
-      <x:c r="R4" s="25" t="str">
+      <x:c r="T4" s="25" t="str">
         <x:v>acceptance_action_selector</x:v>
       </x:c>
-      <x:c r="S4" s="12" t="str">
+      <x:c r="U4" s="12" t="str">
         <x:v>acceptance_evidence</x:v>
       </x:c>
-      <x:c r="T4" s="12" t="str">
+      <x:c r="V4" s="12" t="str">
         <x:v>rejection_path</x:v>
       </x:c>
-      <x:c r="U4" s="25" t="str">
+      <x:c r="W4" s="25" t="str">
         <x:v>return_path</x:v>
       </x:c>
-      <x:c r="V4" s="25" t="str">
+      <x:c r="X4" s="25" t="str">
         <x:v>fallback_path</x:v>
       </x:c>
-      <x:c r="W4" s="12" t="str">
+      <x:c r="Y4" s="12" t="str">
         <x:v>knowledge_status</x:v>
       </x:c>
-      <x:c r="X4" s="12" t="str">
+      <x:c r="Z4" s="12" t="str">
         <x:v>source_id</x:v>
       </x:c>
-      <x:c r="Y4" s="25" t="str">
+      <x:c r="AA4" s="25" t="str">
         <x:v>source_selector</x:v>
       </x:c>
-      <x:c r="Z4" s="25" t="str">
+      <x:c r="AB4" s="25" t="str">
         <x:v>source_locator</x:v>
       </x:c>
-      <x:c r="AA4" s="25" t="str">
+      <x:c r="AC4" s="25" t="str">
         <x:v>last_reviewed</x:v>
       </x:c>
-      <x:c r="AB4" s="25" t="str">
+      <x:c r="AD4" s="25" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -26485,6 +26659,8 @@
       <x:c r="Z5" s="14"/>
       <x:c r="AA5" s="14"/>
       <x:c r="AB5" s="14"/>
+      <x:c r="AC5" s="14"/>
+      <x:c r="AD5" s="14"/>
     </x:row>
     <x:row r="6" ht="16.5" customHeight="1">
       <x:c r="A6" s="14"/>
@@ -26515,6 +26691,8 @@
       <x:c r="Z6" s="14"/>
       <x:c r="AA6" s="14"/>
       <x:c r="AB6" s="14"/>
+      <x:c r="AC6" s="14"/>
+      <x:c r="AD6" s="14"/>
     </x:row>
     <x:row r="7" ht="16.5" customHeight="1">
       <x:c r="A7" s="14"/>
@@ -26545,6 +26723,8 @@
       <x:c r="Z7" s="14"/>
       <x:c r="AA7" s="14"/>
       <x:c r="AB7" s="14"/>
+      <x:c r="AC7" s="14"/>
+      <x:c r="AD7" s="14"/>
     </x:row>
     <x:row r="8" ht="16.5" customHeight="1">
       <x:c r="A8" s="14"/>
@@ -26575,6 +26755,8 @@
       <x:c r="Z8" s="14"/>
       <x:c r="AA8" s="14"/>
       <x:c r="AB8" s="14"/>
+      <x:c r="AC8" s="14"/>
+      <x:c r="AD8" s="14"/>
     </x:row>
     <x:row r="9" ht="16.5" customHeight="1">
       <x:c r="A9" s="14"/>
@@ -26605,6 +26787,8 @@
       <x:c r="Z9" s="14"/>
       <x:c r="AA9" s="14"/>
       <x:c r="AB9" s="14"/>
+      <x:c r="AC9" s="14"/>
+      <x:c r="AD9" s="14"/>
     </x:row>
     <x:row r="10" ht="16.5" customHeight="1">
       <x:c r="A10" s="14"/>
@@ -26635,6 +26819,8 @@
       <x:c r="Z10" s="14"/>
       <x:c r="AA10" s="14"/>
       <x:c r="AB10" s="14"/>
+      <x:c r="AC10" s="14"/>
+      <x:c r="AD10" s="14"/>
     </x:row>
     <x:row r="11" ht="16.5" customHeight="1">
       <x:c r="A11" s="14"/>
@@ -26665,6 +26851,8 @@
       <x:c r="Z11" s="14"/>
       <x:c r="AA11" s="14"/>
       <x:c r="AB11" s="14"/>
+      <x:c r="AC11" s="14"/>
+      <x:c r="AD11" s="14"/>
     </x:row>
     <x:row r="12" ht="16.5" customHeight="1">
       <x:c r="A12" s="14"/>
@@ -26695,6 +26883,8 @@
       <x:c r="Z12" s="14"/>
       <x:c r="AA12" s="14"/>
       <x:c r="AB12" s="14"/>
+      <x:c r="AC12" s="14"/>
+      <x:c r="AD12" s="14"/>
     </x:row>
     <x:row r="13" ht="16.5" customHeight="1">
       <x:c r="A13" s="2"/>
@@ -26725,6 +26915,8 @@
       <x:c r="Z13" s="2"/>
       <x:c r="AA13" s="2"/>
       <x:c r="AB13" s="2"/>
+      <x:c r="AC13" s="2"/>
+      <x:c r="AD13" s="2"/>
     </x:row>
     <x:row r="14" ht="16.5" customHeight="1">
       <x:c r="A14" s="2"/>
@@ -26755,6 +26947,8 @@
       <x:c r="Z14" s="2"/>
       <x:c r="AA14" s="2"/>
       <x:c r="AB14" s="2"/>
+      <x:c r="AC14" s="2"/>
+      <x:c r="AD14" s="2"/>
     </x:row>
     <x:row r="15" ht="16.5" customHeight="1">
       <x:c r="A15" s="2"/>
@@ -26785,6 +26979,8 @@
       <x:c r="Z15" s="2"/>
       <x:c r="AA15" s="2"/>
       <x:c r="AB15" s="2"/>
+      <x:c r="AC15" s="2"/>
+      <x:c r="AD15" s="2"/>
     </x:row>
     <x:row r="16" ht="16.5" customHeight="1">
       <x:c r="A16" s="2"/>
@@ -26815,6 +27011,8 @@
       <x:c r="Z16" s="2"/>
       <x:c r="AA16" s="2"/>
       <x:c r="AB16" s="2"/>
+      <x:c r="AC16" s="2"/>
+      <x:c r="AD16" s="2"/>
     </x:row>
     <x:row r="17" ht="16.5" customHeight="1">
       <x:c r="A17" s="2"/>
@@ -26845,6 +27043,8 @@
       <x:c r="Z17" s="2"/>
       <x:c r="AA17" s="2"/>
       <x:c r="AB17" s="2"/>
+      <x:c r="AC17" s="2"/>
+      <x:c r="AD17" s="2"/>
     </x:row>
     <x:row r="18" ht="16.5" customHeight="1">
       <x:c r="A18" s="2"/>
@@ -26875,6 +27075,8 @@
       <x:c r="Z18" s="2"/>
       <x:c r="AA18" s="2"/>
       <x:c r="AB18" s="2"/>
+      <x:c r="AC18" s="2"/>
+      <x:c r="AD18" s="2"/>
     </x:row>
     <x:row r="19" ht="16.5" customHeight="1">
       <x:c r="A19" s="2"/>
@@ -26905,6 +27107,8 @@
       <x:c r="Z19" s="2"/>
       <x:c r="AA19" s="2"/>
       <x:c r="AB19" s="2"/>
+      <x:c r="AC19" s="2"/>
+      <x:c r="AD19" s="2"/>
     </x:row>
     <x:row r="20" ht="16.5" customHeight="1">
       <x:c r="A20" s="2"/>
@@ -26935,6 +27139,8 @@
       <x:c r="Z20" s="2"/>
       <x:c r="AA20" s="2"/>
       <x:c r="AB20" s="2"/>
+      <x:c r="AC20" s="2"/>
+      <x:c r="AD20" s="2"/>
     </x:row>
     <x:row r="21" ht="16.5" customHeight="1">
       <x:c r="A21" s="2"/>
@@ -26965,6 +27171,8 @@
       <x:c r="Z21" s="2"/>
       <x:c r="AA21" s="2"/>
       <x:c r="AB21" s="2"/>
+      <x:c r="AC21" s="2"/>
+      <x:c r="AD21" s="2"/>
     </x:row>
     <x:row r="22" ht="16.5" customHeight="1">
       <x:c r="A22" s="2"/>
@@ -26995,6 +27203,8 @@
       <x:c r="Z22" s="2"/>
       <x:c r="AA22" s="2"/>
       <x:c r="AB22" s="2"/>
+      <x:c r="AC22" s="2"/>
+      <x:c r="AD22" s="2"/>
     </x:row>
     <x:row r="23" ht="16.5" customHeight="1">
       <x:c r="A23" s="2"/>
@@ -27025,6 +27235,8 @@
       <x:c r="Z23" s="2"/>
       <x:c r="AA23" s="2"/>
       <x:c r="AB23" s="2"/>
+      <x:c r="AC23" s="2"/>
+      <x:c r="AD23" s="2"/>
     </x:row>
     <x:row r="24" ht="16.5" customHeight="1">
       <x:c r="A24" s="2"/>
@@ -27055,6 +27267,8 @@
       <x:c r="Z24" s="2"/>
       <x:c r="AA24" s="2"/>
       <x:c r="AB24" s="2"/>
+      <x:c r="AC24" s="2"/>
+      <x:c r="AD24" s="2"/>
     </x:row>
     <x:row r="25" ht="16.5" customHeight="1">
       <x:c r="A25" s="2"/>
@@ -27085,6 +27299,8 @@
       <x:c r="Z25" s="2"/>
       <x:c r="AA25" s="2"/>
       <x:c r="AB25" s="2"/>
+      <x:c r="AC25" s="2"/>
+      <x:c r="AD25" s="2"/>
     </x:row>
     <x:row r="26" ht="16.5" customHeight="1">
       <x:c r="A26" s="2"/>
@@ -27115,6 +27331,8 @@
       <x:c r="Z26" s="2"/>
       <x:c r="AA26" s="2"/>
       <x:c r="AB26" s="2"/>
+      <x:c r="AC26" s="2"/>
+      <x:c r="AD26" s="2"/>
     </x:row>
     <x:row r="27" ht="16.5" customHeight="1">
       <x:c r="A27" s="2"/>
@@ -27145,6 +27363,8 @@
       <x:c r="Z27" s="2"/>
       <x:c r="AA27" s="2"/>
       <x:c r="AB27" s="2"/>
+      <x:c r="AC27" s="2"/>
+      <x:c r="AD27" s="2"/>
     </x:row>
     <x:row r="28" ht="16.5" customHeight="1">
       <x:c r="A28" s="2"/>
@@ -27175,6 +27395,8 @@
       <x:c r="Z28" s="2"/>
       <x:c r="AA28" s="2"/>
       <x:c r="AB28" s="2"/>
+      <x:c r="AC28" s="2"/>
+      <x:c r="AD28" s="2"/>
     </x:row>
     <x:row r="29" ht="16.5" customHeight="1">
       <x:c r="A29" s="2"/>
@@ -27205,6 +27427,8 @@
       <x:c r="Z29" s="2"/>
       <x:c r="AA29" s="2"/>
       <x:c r="AB29" s="2"/>
+      <x:c r="AC29" s="2"/>
+      <x:c r="AD29" s="2"/>
     </x:row>
     <x:row r="30" ht="16.5" customHeight="1">
       <x:c r="A30" s="2"/>
@@ -27235,6 +27459,8 @@
       <x:c r="Z30" s="2"/>
       <x:c r="AA30" s="2"/>
       <x:c r="AB30" s="2"/>
+      <x:c r="AC30" s="2"/>
+      <x:c r="AD30" s="2"/>
     </x:row>
     <x:row r="31" ht="16.5" customHeight="1">
       <x:c r="A31" s="2"/>
@@ -27265,6 +27491,8 @@
       <x:c r="Z31" s="2"/>
       <x:c r="AA31" s="2"/>
       <x:c r="AB31" s="2"/>
+      <x:c r="AC31" s="2"/>
+      <x:c r="AD31" s="2"/>
     </x:row>
     <x:row r="32" ht="16.5" customHeight="1">
       <x:c r="A32" s="2"/>
@@ -27295,6 +27523,8 @@
       <x:c r="Z32" s="2"/>
       <x:c r="AA32" s="2"/>
       <x:c r="AB32" s="2"/>
+      <x:c r="AC32" s="2"/>
+      <x:c r="AD32" s="2"/>
     </x:row>
     <x:row r="33" ht="16.5" customHeight="1">
       <x:c r="A33" s="2"/>
@@ -27325,6 +27555,8 @@
       <x:c r="Z33" s="2"/>
       <x:c r="AA33" s="2"/>
       <x:c r="AB33" s="2"/>
+      <x:c r="AC33" s="2"/>
+      <x:c r="AD33" s="2"/>
     </x:row>
     <x:row r="34" ht="16.5" customHeight="1">
       <x:c r="A34" s="2"/>
@@ -27355,6 +27587,8 @@
       <x:c r="Z34" s="2"/>
       <x:c r="AA34" s="2"/>
       <x:c r="AB34" s="2"/>
+      <x:c r="AC34" s="2"/>
+      <x:c r="AD34" s="2"/>
     </x:row>
     <x:row r="35" ht="16.5" customHeight="1">
       <x:c r="A35" s="2"/>
@@ -27385,6 +27619,8 @@
       <x:c r="Z35" s="2"/>
       <x:c r="AA35" s="2"/>
       <x:c r="AB35" s="2"/>
+      <x:c r="AC35" s="2"/>
+      <x:c r="AD35" s="2"/>
     </x:row>
     <x:row r="36" ht="16.5" customHeight="1">
       <x:c r="A36" s="2"/>
@@ -27415,6 +27651,8 @@
       <x:c r="Z36" s="2"/>
       <x:c r="AA36" s="2"/>
       <x:c r="AB36" s="2"/>
+      <x:c r="AC36" s="2"/>
+      <x:c r="AD36" s="2"/>
     </x:row>
     <x:row r="37" ht="16.5" customHeight="1">
       <x:c r="A37" s="2"/>
@@ -27445,6 +27683,8 @@
       <x:c r="Z37" s="2"/>
       <x:c r="AA37" s="2"/>
       <x:c r="AB37" s="2"/>
+      <x:c r="AC37" s="2"/>
+      <x:c r="AD37" s="2"/>
     </x:row>
     <x:row r="38" ht="16.5" customHeight="1">
       <x:c r="A38" s="2"/>
@@ -27475,6 +27715,8 @@
       <x:c r="Z38" s="2"/>
       <x:c r="AA38" s="2"/>
       <x:c r="AB38" s="2"/>
+      <x:c r="AC38" s="2"/>
+      <x:c r="AD38" s="2"/>
     </x:row>
     <x:row r="39" ht="16.5" customHeight="1">
       <x:c r="A39" s="2"/>
@@ -27505,6 +27747,8 @@
       <x:c r="Z39" s="2"/>
       <x:c r="AA39" s="2"/>
       <x:c r="AB39" s="2"/>
+      <x:c r="AC39" s="2"/>
+      <x:c r="AD39" s="2"/>
     </x:row>
     <x:row r="40" ht="16.5" customHeight="1">
       <x:c r="A40" s="2"/>
@@ -27535,6 +27779,8 @@
       <x:c r="Z40" s="2"/>
       <x:c r="AA40" s="2"/>
       <x:c r="AB40" s="2"/>
+      <x:c r="AC40" s="2"/>
+      <x:c r="AD40" s="2"/>
     </x:row>
     <x:row r="41" ht="16.5" customHeight="1">
       <x:c r="A41" s="2"/>
@@ -27565,6 +27811,8 @@
       <x:c r="Z41" s="2"/>
       <x:c r="AA41" s="2"/>
       <x:c r="AB41" s="2"/>
+      <x:c r="AC41" s="2"/>
+      <x:c r="AD41" s="2"/>
     </x:row>
     <x:row r="42" ht="16.5" customHeight="1">
       <x:c r="A42" s="2"/>
@@ -27595,6 +27843,8 @@
       <x:c r="Z42" s="2"/>
       <x:c r="AA42" s="2"/>
       <x:c r="AB42" s="2"/>
+      <x:c r="AC42" s="2"/>
+      <x:c r="AD42" s="2"/>
     </x:row>
     <x:row r="43" ht="16.5" customHeight="1">
       <x:c r="A43" s="2"/>
@@ -27625,6 +27875,8 @@
       <x:c r="Z43" s="2"/>
       <x:c r="AA43" s="2"/>
       <x:c r="AB43" s="2"/>
+      <x:c r="AC43" s="2"/>
+      <x:c r="AD43" s="2"/>
     </x:row>
     <x:row r="44" ht="16.5" customHeight="1">
       <x:c r="A44" s="2"/>
@@ -27655,6 +27907,8 @@
       <x:c r="Z44" s="2"/>
       <x:c r="AA44" s="2"/>
       <x:c r="AB44" s="2"/>
+      <x:c r="AC44" s="2"/>
+      <x:c r="AD44" s="2"/>
     </x:row>
     <x:row r="45" ht="16.5" customHeight="1">
       <x:c r="A45" s="2"/>
@@ -27685,6 +27939,8 @@
       <x:c r="Z45" s="2"/>
       <x:c r="AA45" s="2"/>
       <x:c r="AB45" s="2"/>
+      <x:c r="AC45" s="2"/>
+      <x:c r="AD45" s="2"/>
     </x:row>
     <x:row r="46" ht="16.5" customHeight="1">
       <x:c r="A46" s="2"/>
@@ -27715,6 +27971,8 @@
       <x:c r="Z46" s="2"/>
       <x:c r="AA46" s="2"/>
       <x:c r="AB46" s="2"/>
+      <x:c r="AC46" s="2"/>
+      <x:c r="AD46" s="2"/>
     </x:row>
     <x:row r="47" ht="16.5" customHeight="1">
       <x:c r="A47" s="2"/>
@@ -27745,6 +28003,8 @@
       <x:c r="Z47" s="2"/>
       <x:c r="AA47" s="2"/>
       <x:c r="AB47" s="2"/>
+      <x:c r="AC47" s="2"/>
+      <x:c r="AD47" s="2"/>
     </x:row>
     <x:row r="48" ht="16.5" customHeight="1">
       <x:c r="A48" s="2"/>
@@ -27775,6 +28035,8 @@
       <x:c r="Z48" s="2"/>
       <x:c r="AA48" s="2"/>
       <x:c r="AB48" s="2"/>
+      <x:c r="AC48" s="2"/>
+      <x:c r="AD48" s="2"/>
     </x:row>
     <x:row r="49" ht="16.5" customHeight="1">
       <x:c r="A49" s="2"/>
@@ -27805,6 +28067,8 @@
       <x:c r="Z49" s="2"/>
       <x:c r="AA49" s="2"/>
       <x:c r="AB49" s="2"/>
+      <x:c r="AC49" s="2"/>
+      <x:c r="AD49" s="2"/>
     </x:row>
     <x:row r="50" ht="16.5" customHeight="1">
       <x:c r="A50" s="2"/>
@@ -27835,6 +28099,8 @@
       <x:c r="Z50" s="2"/>
       <x:c r="AA50" s="2"/>
       <x:c r="AB50" s="2"/>
+      <x:c r="AC50" s="2"/>
+      <x:c r="AD50" s="2"/>
     </x:row>
     <x:row r="51" ht="16.5" customHeight="1">
       <x:c r="A51" s="2"/>
@@ -27865,6 +28131,8 @@
       <x:c r="Z51" s="2"/>
       <x:c r="AA51" s="2"/>
       <x:c r="AB51" s="2"/>
+      <x:c r="AC51" s="2"/>
+      <x:c r="AD51" s="2"/>
     </x:row>
     <x:row r="52" ht="16.5" customHeight="1">
       <x:c r="A52" s="2"/>
@@ -27895,6 +28163,8 @@
       <x:c r="Z52" s="2"/>
       <x:c r="AA52" s="2"/>
       <x:c r="AB52" s="2"/>
+      <x:c r="AC52" s="2"/>
+      <x:c r="AD52" s="2"/>
     </x:row>
     <x:row r="53" ht="16.5" customHeight="1">
       <x:c r="A53" s="2"/>
@@ -27925,6 +28195,8 @@
       <x:c r="Z53" s="2"/>
       <x:c r="AA53" s="2"/>
       <x:c r="AB53" s="2"/>
+      <x:c r="AC53" s="2"/>
+      <x:c r="AD53" s="2"/>
     </x:row>
     <x:row r="54" ht="16.5" customHeight="1">
       <x:c r="A54" s="2"/>
@@ -27955,6 +28227,8 @@
       <x:c r="Z54" s="2"/>
       <x:c r="AA54" s="2"/>
       <x:c r="AB54" s="2"/>
+      <x:c r="AC54" s="2"/>
+      <x:c r="AD54" s="2"/>
     </x:row>
     <x:row r="55" ht="16.5" customHeight="1">
       <x:c r="A55" s="2"/>
@@ -27985,6 +28259,8 @@
       <x:c r="Z55" s="2"/>
       <x:c r="AA55" s="2"/>
       <x:c r="AB55" s="2"/>
+      <x:c r="AC55" s="2"/>
+      <x:c r="AD55" s="2"/>
     </x:row>
     <x:row r="56" ht="16.5" customHeight="1">
       <x:c r="A56" s="2"/>
@@ -28015,6 +28291,8 @@
       <x:c r="Z56" s="2"/>
       <x:c r="AA56" s="2"/>
       <x:c r="AB56" s="2"/>
+      <x:c r="AC56" s="2"/>
+      <x:c r="AD56" s="2"/>
     </x:row>
     <x:row r="57" ht="16.5" customHeight="1">
       <x:c r="A57" s="2"/>
@@ -28045,6 +28323,8 @@
       <x:c r="Z57" s="2"/>
       <x:c r="AA57" s="2"/>
       <x:c r="AB57" s="2"/>
+      <x:c r="AC57" s="2"/>
+      <x:c r="AD57" s="2"/>
     </x:row>
     <x:row r="58" ht="16.5" customHeight="1">
       <x:c r="A58" s="2"/>
@@ -28075,6 +28355,8 @@
       <x:c r="Z58" s="2"/>
       <x:c r="AA58" s="2"/>
       <x:c r="AB58" s="2"/>
+      <x:c r="AC58" s="2"/>
+      <x:c r="AD58" s="2"/>
     </x:row>
     <x:row r="59" ht="16.5" customHeight="1">
       <x:c r="A59" s="2"/>
@@ -28105,6 +28387,8 @@
       <x:c r="Z59" s="2"/>
       <x:c r="AA59" s="2"/>
       <x:c r="AB59" s="2"/>
+      <x:c r="AC59" s="2"/>
+      <x:c r="AD59" s="2"/>
     </x:row>
     <x:row r="60" ht="16.5" customHeight="1">
       <x:c r="A60" s="2"/>
@@ -28135,6 +28419,8 @@
       <x:c r="Z60" s="2"/>
       <x:c r="AA60" s="2"/>
       <x:c r="AB60" s="2"/>
+      <x:c r="AC60" s="2"/>
+      <x:c r="AD60" s="2"/>
     </x:row>
     <x:row r="61" ht="16.5" customHeight="1">
       <x:c r="A61" s="2"/>
@@ -28165,6 +28451,8 @@
       <x:c r="Z61" s="2"/>
       <x:c r="AA61" s="2"/>
       <x:c r="AB61" s="2"/>
+      <x:c r="AC61" s="2"/>
+      <x:c r="AD61" s="2"/>
     </x:row>
     <x:row r="62" ht="16.5" customHeight="1">
       <x:c r="A62" s="2"/>
@@ -28195,6 +28483,8 @@
       <x:c r="Z62" s="2"/>
       <x:c r="AA62" s="2"/>
       <x:c r="AB62" s="2"/>
+      <x:c r="AC62" s="2"/>
+      <x:c r="AD62" s="2"/>
     </x:row>
     <x:row r="63" ht="16.5" customHeight="1">
       <x:c r="A63" s="2"/>
@@ -28225,6 +28515,8 @@
       <x:c r="Z63" s="2"/>
       <x:c r="AA63" s="2"/>
       <x:c r="AB63" s="2"/>
+      <x:c r="AC63" s="2"/>
+      <x:c r="AD63" s="2"/>
     </x:row>
     <x:row r="64" ht="16.5" customHeight="1">
       <x:c r="A64" s="2"/>
@@ -28255,6 +28547,8 @@
       <x:c r="Z64" s="2"/>
       <x:c r="AA64" s="2"/>
       <x:c r="AB64" s="2"/>
+      <x:c r="AC64" s="2"/>
+      <x:c r="AD64" s="2"/>
     </x:row>
     <x:row r="65" ht="16.5" customHeight="1">
       <x:c r="A65" s="2"/>
@@ -28285,6 +28579,8 @@
       <x:c r="Z65" s="2"/>
       <x:c r="AA65" s="2"/>
       <x:c r="AB65" s="2"/>
+      <x:c r="AC65" s="2"/>
+      <x:c r="AD65" s="2"/>
     </x:row>
     <x:row r="66" ht="16.5" customHeight="1">
       <x:c r="A66" s="2"/>
@@ -28315,6 +28611,8 @@
       <x:c r="Z66" s="2"/>
       <x:c r="AA66" s="2"/>
       <x:c r="AB66" s="2"/>
+      <x:c r="AC66" s="2"/>
+      <x:c r="AD66" s="2"/>
     </x:row>
     <x:row r="67" ht="16.5" customHeight="1">
       <x:c r="A67" s="2"/>
@@ -28345,6 +28643,8 @@
       <x:c r="Z67" s="2"/>
       <x:c r="AA67" s="2"/>
       <x:c r="AB67" s="2"/>
+      <x:c r="AC67" s="2"/>
+      <x:c r="AD67" s="2"/>
     </x:row>
     <x:row r="68" ht="16.5" customHeight="1">
       <x:c r="A68" s="2"/>
@@ -28375,6 +28675,8 @@
       <x:c r="Z68" s="2"/>
       <x:c r="AA68" s="2"/>
       <x:c r="AB68" s="2"/>
+      <x:c r="AC68" s="2"/>
+      <x:c r="AD68" s="2"/>
     </x:row>
     <x:row r="69" ht="16.5" customHeight="1">
       <x:c r="A69" s="2"/>
@@ -28405,6 +28707,8 @@
       <x:c r="Z69" s="2"/>
       <x:c r="AA69" s="2"/>
       <x:c r="AB69" s="2"/>
+      <x:c r="AC69" s="2"/>
+      <x:c r="AD69" s="2"/>
     </x:row>
     <x:row r="70" ht="16.5" customHeight="1">
       <x:c r="A70" s="2"/>
@@ -28435,6 +28739,8 @@
       <x:c r="Z70" s="2"/>
       <x:c r="AA70" s="2"/>
       <x:c r="AB70" s="2"/>
+      <x:c r="AC70" s="2"/>
+      <x:c r="AD70" s="2"/>
     </x:row>
     <x:row r="71" ht="16.5" customHeight="1">
       <x:c r="A71" s="2"/>
@@ -28465,6 +28771,8 @@
       <x:c r="Z71" s="2"/>
       <x:c r="AA71" s="2"/>
       <x:c r="AB71" s="2"/>
+      <x:c r="AC71" s="2"/>
+      <x:c r="AD71" s="2"/>
     </x:row>
     <x:row r="72" ht="16.5" customHeight="1">
       <x:c r="A72" s="2"/>
@@ -28495,6 +28803,8 @@
       <x:c r="Z72" s="2"/>
       <x:c r="AA72" s="2"/>
       <x:c r="AB72" s="2"/>
+      <x:c r="AC72" s="2"/>
+      <x:c r="AD72" s="2"/>
     </x:row>
     <x:row r="73" ht="16.5" customHeight="1">
       <x:c r="A73" s="2"/>
@@ -28525,6 +28835,8 @@
       <x:c r="Z73" s="2"/>
       <x:c r="AA73" s="2"/>
       <x:c r="AB73" s="2"/>
+      <x:c r="AC73" s="2"/>
+      <x:c r="AD73" s="2"/>
     </x:row>
     <x:row r="74" ht="16.5" customHeight="1">
       <x:c r="A74" s="2"/>
@@ -28555,6 +28867,8 @@
       <x:c r="Z74" s="2"/>
       <x:c r="AA74" s="2"/>
       <x:c r="AB74" s="2"/>
+      <x:c r="AC74" s="2"/>
+      <x:c r="AD74" s="2"/>
     </x:row>
     <x:row r="75" ht="16.5" customHeight="1">
       <x:c r="A75" s="2"/>
@@ -28585,6 +28899,8 @@
       <x:c r="Z75" s="2"/>
       <x:c r="AA75" s="2"/>
       <x:c r="AB75" s="2"/>
+      <x:c r="AC75" s="2"/>
+      <x:c r="AD75" s="2"/>
     </x:row>
     <x:row r="76" ht="16.5" customHeight="1">
       <x:c r="A76" s="2"/>
@@ -28615,6 +28931,8 @@
       <x:c r="Z76" s="2"/>
       <x:c r="AA76" s="2"/>
       <x:c r="AB76" s="2"/>
+      <x:c r="AC76" s="2"/>
+      <x:c r="AD76" s="2"/>
     </x:row>
     <x:row r="77" ht="16.5" customHeight="1">
       <x:c r="A77" s="2"/>
@@ -28645,6 +28963,8 @@
       <x:c r="Z77" s="2"/>
       <x:c r="AA77" s="2"/>
       <x:c r="AB77" s="2"/>
+      <x:c r="AC77" s="2"/>
+      <x:c r="AD77" s="2"/>
     </x:row>
     <x:row r="78" ht="16.5" customHeight="1">
       <x:c r="A78" s="2"/>
@@ -28675,6 +28995,8 @@
       <x:c r="Z78" s="2"/>
       <x:c r="AA78" s="2"/>
       <x:c r="AB78" s="2"/>
+      <x:c r="AC78" s="2"/>
+      <x:c r="AD78" s="2"/>
     </x:row>
     <x:row r="79" ht="16.5" customHeight="1">
       <x:c r="A79" s="2"/>
@@ -28705,6 +29027,8 @@
       <x:c r="Z79" s="2"/>
       <x:c r="AA79" s="2"/>
       <x:c r="AB79" s="2"/>
+      <x:c r="AC79" s="2"/>
+      <x:c r="AD79" s="2"/>
     </x:row>
     <x:row r="80" ht="16.5" customHeight="1">
       <x:c r="A80" s="2"/>
@@ -28735,6 +29059,8 @@
       <x:c r="Z80" s="2"/>
       <x:c r="AA80" s="2"/>
       <x:c r="AB80" s="2"/>
+      <x:c r="AC80" s="2"/>
+      <x:c r="AD80" s="2"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -51811,7 +52137,7 @@
         <x:v>направление</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>продукт</x:v>
+        <x:v>компонент</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
         <x:v>контракт</x:v>
@@ -51866,7 +52192,7 @@
         <x:v>поставляет</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>Лид качества A</x:v>
+        <x:v>Лид качества A (продукт)</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
         <x:v>Поставка лидов</x:v>

</xml_diff>

<commit_message>
release: publish production-system skills v0.3
</commit_message>
<xml_diff>
--- a/outputs/v0.3-review/production-system-model-template-v0.3-review.xlsx
+++ b/outputs/v0.3-review/production-system-model-template-v0.3-review.xlsx
@@ -2,38 +2,38 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="R83d98d95285f4652"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Система" sheetId="2" r:id="R16fd2f9b0a3446e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Схема шаблона" sheetId="3" r:id="Re5818f0deadd45ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="4" r:id="Rfba858c3fd364450"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версии" sheetId="5" r:id="R9d70a2599d6148ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исполнители" sheetId="6" r:id="R8951b197abb04acd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции" sheetId="7" r:id="Rb09807b6e16b43ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Назначения" sheetId="8" r:id="Rc998c3d6282f453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контрагенты" sheetId="9" r:id="R0dbcf0e2e2fd4a6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Продукты" sheetId="10" r:id="R09a3dd813b7e48a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Материалы" sheetId="11" r:id="R0741307f26234d77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процессы" sheetId="12" r:id="R65bf3039b10845ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действия" sheetId="13" r:id="R8b4382e373254675"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи действий" sheetId="14" r:id="R56d696007720493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объекты" sheetId="15" r:id="Raa6f64bb8d62445a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Состояния" sheetId="16" r:id="R497d067597784ed7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переходы" sheetId="17" r:id="R48200412d3104296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Элементы модели" sheetId="18" r:id="Rc81163db643f4c43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контракты" sheetId="19" r:id="R05ef3011615b42d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции контрактов" sheetId="20" r:id="Rac4f35883ef646cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Интерфейсы передачи" sheetId="21" r:id="R948cfd217bd4434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи модели" sheetId="22" r:id="R689c2c12123d4bf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Решения" sheetId="23" r:id="R0fa9c976e6fb4cf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения модели" sheetId="24" r:id="R066a4760796345a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отклонения" sheetId="25" r:id="Rb2b5ecff5e004c7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гипотезы" sheetId="26" r:id="Rdeb43baaa5834cb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперименты" sheetId="27" r:id="Rf152118680944575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез модели" sheetId="28" r:id="Ra16cb255e9ff4245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Проверки" sheetId="29" r:id="Rd5c0ac14d8ab49b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр процессов" sheetId="30" r:id="R1ef8fb0ed23948c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Рабочая панель" sheetId="31" r:id="Re5c398211e094101"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Диаграммы" sheetId="32" r:id="R191ac82d7c2544e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" r:id="Rcf0097c2d28245e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Система" sheetId="2" r:id="R54d3e04a4a034561"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Схема шаблона" sheetId="3" r:id="R1ca2966665e248d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="4" r:id="R291ac5e23fa245e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Версии" sheetId="5" r:id="R95d4097c2da54c34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Исполнители" sheetId="6" r:id="R97e2a66fac19410f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции" sheetId="7" r:id="Rdb9ed97c859641f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Назначения" sheetId="8" r:id="R6fbd485381934e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контрагенты" sheetId="9" r:id="Rb38a67ceb566453d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Продукты" sheetId="10" r:id="Rdd8b2de4d1cd434c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Материалы" sheetId="11" r:id="R528e139af29748bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Процессы" sheetId="12" r:id="R6bb0e39f9bc34039"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Действия" sheetId="13" r:id="R28fa990f51fc4162"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи действий" sheetId="14" r:id="Rd53776f5b9b344ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Объекты" sheetId="15" r:id="Rab20077a778c42ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Состояния" sheetId="16" r:id="R02a4244c7f8d4e20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переходы" sheetId="17" r:id="R41eba97d67a945b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Элементы модели" sheetId="18" r:id="R177dce8b62af4670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Контракты" sheetId="19" r:id="R6c663c2927b740e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Позиции контрактов" sheetId="20" r:id="R5e0566859a954583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Интерфейсы передачи" sheetId="21" r:id="Rb082c163432e4258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Связи модели" sheetId="22" r:id="R3e6b4cbfa15e4cfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Решения" sheetId="23" r:id="R8a22cffc98584f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Изменения модели" sheetId="24" r:id="R2bce757ac00b4d4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Отклонения" sheetId="25" r:id="R1be572c044684786"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гипотезы" sheetId="26" r:id="Ra4a3521783024961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперименты" sheetId="27" r:id="R1b71706679d44cce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Срез модели" sheetId="28" r:id="R81bf9d4b427b43dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Проверки" sheetId="29" r:id="R183515bd997e452c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр процессов" sheetId="30" r:id="Red14786c5f6046a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Рабочая панель" sheetId="31" r:id="Rfea9a2bb518b4dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Диаграммы" sheetId="32" r:id="R03e642338ca24e21"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="enum_yes_no">'Система'!BA2:BA3</x:definedName>

</xml_diff>